<commit_message>
changed the timer so that it rounds to the nearest 30 minutes rather than going to the original 3 times of 8AM, 11AM, and 2:30PM.
</commit_message>
<xml_diff>
--- a/Select_Menu_Patient_Log.xlsx
+++ b/Select_Menu_Patient_Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dvagov-my.sharepoint.com/personal/crystal_alvarez_va_gov/Documents/Desktop/Select Menu/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dvagov-my.sharepoint.com/personal/crystal_alvarez_va_gov/Documents/Desktop/Select Menu/VSCode/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="447" documentId="13_ncr:1_{9CEB82FD-F55C-4572-8711-23C7E1DF9E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F446DD70-4435-4FF5-90E2-EA24888A5648}"/>
+  <xr:revisionPtr revIDLastSave="606" documentId="13_ncr:1_{9CEB82FD-F55C-4572-8711-23C7E1DF9E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFF5F4CA-6A48-42AF-BB31-F541AA70F24A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient_Log" sheetId="1" r:id="rId1"/>
@@ -168,7 +168,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2714" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2997" uniqueCount="477">
   <si>
     <t>Date</t>
   </si>
@@ -1491,6 +1491,114 @@
   </si>
   <si>
     <t>5:00 PM</t>
+  </si>
+  <si>
+    <t>SLEEPING CHOSE MEAL FOR HIM</t>
+  </si>
+  <si>
+    <t>Patient says veggies are not cooked enough and brussels sprouts were too dry.</t>
+  </si>
+  <si>
+    <t>6:30 PM</t>
+  </si>
+  <si>
+    <t>AIRBORNE PRECAUTION CHOSE MAIN MEAL MINUS DISLIKES OF CHOLULA</t>
+  </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>D06</t>
+  </si>
+  <si>
+    <t>icu - 3</t>
+  </si>
+  <si>
+    <t>3A31</t>
+  </si>
+  <si>
+    <t>patient wants more hot cereal with breakfast</t>
+  </si>
+  <si>
+    <t>wants a softer diet</t>
+  </si>
+  <si>
+    <t>2c14</t>
+  </si>
+  <si>
+    <t>cannot enter room</t>
+  </si>
+  <si>
+    <t>5:30 PM</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
+  </si>
+  <si>
+    <t>2026-09-26</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>2026-09-19</t>
+  </si>
+  <si>
+    <t>2026-09-20</t>
+  </si>
+  <si>
+    <t>2026-09-17</t>
+  </si>
+  <si>
+    <t>2026-09-12</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
+  </si>
+  <si>
+    <t>2026-09-10</t>
+  </si>
+  <si>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>2026-08-29</t>
+  </si>
+  <si>
+    <t>2026-08-30</t>
+  </si>
+  <si>
+    <t>2026-08-23</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>5.32</t>
+  </si>
+  <si>
+    <t>Pt mentioned being vegetarian but has not seen RD. Decided to not move forward w/ selection process</t>
+  </si>
+  <si>
+    <t>4.97</t>
+  </si>
+  <si>
+    <t>pt did not receive items on "Center" of ticket</t>
+  </si>
+  <si>
+    <t>10.32</t>
+  </si>
+  <si>
+    <t>reviewed dislikes</t>
+  </si>
+  <si>
+    <t>12:00 PM</t>
+  </si>
+  <si>
+    <t>25.86</t>
+  </si>
+  <si>
+    <t>9.20</t>
   </si>
 </sst>
 </file>
@@ -1973,7 +2081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H370"/>
+  <dimension ref="A1:H394"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -1983,6 +2091,7 @@
     <col min="5" max="5" width="10.83203125" style="12" customWidth="1"/>
     <col min="6" max="6" width="21.08203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -3860,8 +3969,8 @@
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A80" s="8">
-        <v>46257</v>
+      <c r="A80" t="s">
+        <v>466</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>18</v>
@@ -3881,8 +3990,8 @@
       <c r="G80" s="10"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A81" s="9">
-        <v>46257</v>
+      <c r="A81" t="s">
+        <v>466</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>18</v>
@@ -3902,8 +4011,8 @@
       <c r="G81" s="10"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A82" s="9">
-        <v>46257</v>
+      <c r="A82" t="s">
+        <v>466</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>18</v>
@@ -3923,8 +4032,8 @@
       <c r="G82" s="10"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A83" s="9">
-        <v>46257</v>
+      <c r="A83" t="s">
+        <v>466</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>18</v>
@@ -3944,8 +4053,8 @@
       <c r="G83" s="10"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A84" s="9">
-        <v>46257</v>
+      <c r="A84" t="s">
+        <v>466</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>10</v>
@@ -3968,8 +4077,8 @@
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A85" s="9">
-        <v>46257</v>
+      <c r="A85" t="s">
+        <v>466</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>18</v>
@@ -3989,8 +4098,8 @@
       <c r="G85" s="10"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A86" s="9">
-        <v>46257</v>
+      <c r="A86" t="s">
+        <v>466</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>18</v>
@@ -4010,8 +4119,8 @@
       <c r="G86" s="10"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A87" s="9">
-        <v>46257</v>
+      <c r="A87" t="s">
+        <v>466</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>18</v>
@@ -4034,8 +4143,8 @@
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A88" s="9">
-        <v>46257</v>
+      <c r="A88" t="s">
+        <v>466</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>18</v>
@@ -4055,8 +4164,8 @@
       <c r="G88" s="10"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A89" s="9">
-        <v>46257</v>
+      <c r="A89" t="s">
+        <v>466</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>10</v>
@@ -4620,8 +4729,8 @@
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A113" s="9">
-        <v>46259</v>
+      <c r="A113" t="s">
+        <v>160</v>
       </c>
       <c r="B113" s="10" t="s">
         <v>18</v>
@@ -4640,8 +4749,8 @@
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A114" s="9">
-        <v>46259</v>
+      <c r="A114" t="s">
+        <v>160</v>
       </c>
       <c r="B114" s="10" t="s">
         <v>18</v>
@@ -4976,8 +5085,8 @@
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A129" s="8">
-        <v>46261</v>
+      <c r="A129" t="s">
+        <v>180</v>
       </c>
       <c r="B129" t="s">
         <v>10</v>
@@ -4996,8 +5105,8 @@
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A130" s="8">
-        <v>46261</v>
+      <c r="A130" t="s">
+        <v>180</v>
       </c>
       <c r="B130" t="s">
         <v>10</v>
@@ -5016,8 +5125,8 @@
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A131" s="8">
-        <v>46261</v>
+      <c r="A131" t="s">
+        <v>180</v>
       </c>
       <c r="B131" t="s">
         <v>10</v>
@@ -5039,8 +5148,8 @@
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A132" s="8">
-        <v>46261</v>
+      <c r="A132" t="s">
+        <v>180</v>
       </c>
       <c r="B132" s="10" t="s">
         <v>18</v>
@@ -5060,8 +5169,8 @@
       <c r="G132" s="10"/>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A133" s="8">
-        <v>46261</v>
+      <c r="A133" t="s">
+        <v>180</v>
       </c>
       <c r="B133" s="10" t="s">
         <v>18</v>
@@ -5084,8 +5193,8 @@
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A134" s="8">
-        <v>46261</v>
+      <c r="A134" t="s">
+        <v>180</v>
       </c>
       <c r="B134" s="10" t="s">
         <v>18</v>
@@ -5108,8 +5217,8 @@
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A135" s="8">
-        <v>46261</v>
+      <c r="A135" t="s">
+        <v>180</v>
       </c>
       <c r="B135" s="10" t="s">
         <v>18</v>
@@ -5132,8 +5241,8 @@
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A136" s="8">
-        <v>46261</v>
+      <c r="A136" t="s">
+        <v>180</v>
       </c>
       <c r="B136" s="10" t="s">
         <v>18</v>
@@ -5156,8 +5265,8 @@
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A137" s="8">
-        <v>46261</v>
+      <c r="A137" t="s">
+        <v>180</v>
       </c>
       <c r="B137" s="10" t="s">
         <v>18</v>
@@ -5177,8 +5286,8 @@
       <c r="G137" s="10"/>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A138" s="8">
-        <v>46261</v>
+      <c r="A138" t="s">
+        <v>180</v>
       </c>
       <c r="B138" s="10" t="s">
         <v>18</v>
@@ -5198,8 +5307,8 @@
       <c r="G138" s="10"/>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A139" s="9">
-        <v>46262</v>
+      <c r="A139" t="s">
+        <v>463</v>
       </c>
       <c r="B139" s="10" t="s">
         <v>10</v>
@@ -5219,8 +5328,8 @@
       <c r="G139" s="10"/>
     </row>
     <row r="140" spans="1:8" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A140" s="9">
-        <v>46262</v>
+      <c r="A140" t="s">
+        <v>463</v>
       </c>
       <c r="B140" s="10" t="s">
         <v>10</v>
@@ -5243,8 +5352,8 @@
       </c>
     </row>
     <row r="141" spans="1:8" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A141" s="9">
-        <v>46262</v>
+      <c r="A141" t="s">
+        <v>463</v>
       </c>
       <c r="B141" s="10" t="s">
         <v>18</v>
@@ -5267,8 +5376,8 @@
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A142" s="9">
-        <v>46262</v>
+      <c r="A142" t="s">
+        <v>463</v>
       </c>
       <c r="B142" s="10" t="s">
         <v>18</v>
@@ -5288,8 +5397,8 @@
       <c r="G142" s="10"/>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A143" s="9">
-        <v>46262</v>
+      <c r="A143" t="s">
+        <v>463</v>
       </c>
       <c r="B143" s="10" t="s">
         <v>18</v>
@@ -5309,8 +5418,8 @@
       <c r="G143" s="10"/>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A144" s="9">
-        <v>46262</v>
+      <c r="A144" t="s">
+        <v>463</v>
       </c>
       <c r="B144" s="10" t="s">
         <v>18</v>
@@ -5333,8 +5442,8 @@
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A145" s="9">
-        <v>46262</v>
+      <c r="A145" t="s">
+        <v>463</v>
       </c>
       <c r="B145" s="10" t="s">
         <v>18</v>
@@ -5357,8 +5466,8 @@
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A146" s="9">
-        <v>46262</v>
+      <c r="A146" t="s">
+        <v>463</v>
       </c>
       <c r="B146" s="10" t="s">
         <v>10</v>
@@ -5381,8 +5490,8 @@
       </c>
     </row>
     <row r="147" spans="1:8" ht="31" x14ac:dyDescent="0.35">
-      <c r="A147" s="9">
-        <v>46262</v>
+      <c r="A147" t="s">
+        <v>463</v>
       </c>
       <c r="B147" s="10" t="s">
         <v>10</v>
@@ -5404,8 +5513,8 @@
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A148" s="9">
-        <v>46262</v>
+      <c r="A148" t="s">
+        <v>463</v>
       </c>
       <c r="B148" s="10" t="s">
         <v>10</v>
@@ -5425,8 +5534,8 @@
       <c r="G148" s="10"/>
     </row>
     <row r="149" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A149" s="9">
-        <v>46262</v>
+      <c r="A149" t="s">
+        <v>463</v>
       </c>
       <c r="B149" s="10" t="s">
         <v>18</v>
@@ -5449,8 +5558,8 @@
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A150" s="9">
-        <v>46263</v>
+      <c r="A150" t="s">
+        <v>464</v>
       </c>
       <c r="B150" s="10" t="s">
         <v>18</v>
@@ -5470,8 +5579,8 @@
       <c r="G150" s="10"/>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A151" s="9">
-        <v>46263</v>
+      <c r="A151" t="s">
+        <v>464</v>
       </c>
       <c r="B151" s="10" t="s">
         <v>18</v>
@@ -5494,8 +5603,8 @@
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A152" s="9">
-        <v>46263</v>
+      <c r="A152" t="s">
+        <v>464</v>
       </c>
       <c r="B152" s="10" t="s">
         <v>18</v>
@@ -5518,8 +5627,8 @@
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A153" s="9">
-        <v>46263</v>
+      <c r="A153" t="s">
+        <v>464</v>
       </c>
       <c r="B153" s="10" t="s">
         <v>18</v>
@@ -5539,8 +5648,8 @@
       <c r="G153" s="10"/>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A154" s="9">
-        <v>46263</v>
+      <c r="A154" t="s">
+        <v>464</v>
       </c>
       <c r="B154" s="10" t="s">
         <v>18</v>
@@ -5560,8 +5669,8 @@
       <c r="G154" s="10"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A155" s="9">
-        <v>46263</v>
+      <c r="A155" t="s">
+        <v>464</v>
       </c>
       <c r="B155" s="10" t="s">
         <v>18</v>
@@ -5581,8 +5690,8 @@
       <c r="G155" s="10"/>
     </row>
     <row r="156" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A156" s="9">
-        <v>46263</v>
+      <c r="A156" t="s">
+        <v>464</v>
       </c>
       <c r="B156" s="10" t="s">
         <v>10</v>
@@ -5604,8 +5713,8 @@
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A157" s="9">
-        <v>46263</v>
+      <c r="A157" t="s">
+        <v>464</v>
       </c>
       <c r="B157" s="10" t="s">
         <v>10</v>
@@ -5625,8 +5734,8 @@
       <c r="G157" s="10"/>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A158" s="9">
-        <v>46263</v>
+      <c r="A158" t="s">
+        <v>464</v>
       </c>
       <c r="B158" s="10" t="s">
         <v>10</v>
@@ -5646,8 +5755,8 @@
       <c r="G158" s="10"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A159" s="9">
-        <v>46264</v>
+      <c r="A159" t="s">
+        <v>465</v>
       </c>
       <c r="B159" s="10" t="s">
         <v>10</v>
@@ -5670,8 +5779,8 @@
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A160" s="9">
-        <v>46264</v>
+      <c r="A160" t="s">
+        <v>465</v>
       </c>
       <c r="B160" s="10" t="s">
         <v>10</v>
@@ -5691,8 +5800,8 @@
       <c r="G160" s="10"/>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A161" s="9">
-        <v>46264</v>
+      <c r="A161" t="s">
+        <v>465</v>
       </c>
       <c r="B161" s="10" t="s">
         <v>10</v>
@@ -5715,8 +5824,8 @@
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A162" s="9">
-        <v>46264</v>
+      <c r="A162" t="s">
+        <v>465</v>
       </c>
       <c r="B162" s="10" t="s">
         <v>10</v>
@@ -5739,8 +5848,8 @@
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A163" s="9">
-        <v>46264</v>
+      <c r="A163" t="s">
+        <v>465</v>
       </c>
       <c r="B163" s="10" t="s">
         <v>18</v>
@@ -5760,8 +5869,8 @@
       <c r="G163" s="10"/>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A164" s="9">
-        <v>46264</v>
+      <c r="A164" t="s">
+        <v>465</v>
       </c>
       <c r="B164" s="10" t="s">
         <v>18</v>
@@ -5781,8 +5890,8 @@
       <c r="G164" s="10"/>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A165" s="9">
-        <v>46264</v>
+      <c r="A165" t="s">
+        <v>465</v>
       </c>
       <c r="B165" s="10" t="s">
         <v>10</v>
@@ -5805,8 +5914,8 @@
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A166" s="9">
-        <v>46264</v>
+      <c r="A166" t="s">
+        <v>465</v>
       </c>
       <c r="B166" s="10" t="s">
         <v>10</v>
@@ -5826,8 +5935,8 @@
       <c r="G166" s="10"/>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A167" s="9">
-        <v>46264</v>
+      <c r="A167" t="s">
+        <v>465</v>
       </c>
       <c r="B167" s="10" t="s">
         <v>10</v>
@@ -5850,8 +5959,8 @@
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A168" s="9">
-        <v>46264</v>
+      <c r="A168" t="s">
+        <v>465</v>
       </c>
       <c r="B168" s="10" t="s">
         <v>10</v>
@@ -5874,8 +5983,8 @@
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A169" s="9">
-        <v>46264</v>
+      <c r="A169" t="s">
+        <v>465</v>
       </c>
       <c r="B169" s="10" t="s">
         <v>18</v>
@@ -5895,8 +6004,8 @@
       <c r="G169" s="10"/>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A170" s="9">
-        <v>46264</v>
+      <c r="A170" t="s">
+        <v>465</v>
       </c>
       <c r="B170" s="10" t="s">
         <v>18</v>
@@ -5916,8 +6025,8 @@
       <c r="G170" s="10"/>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A171" s="9">
-        <v>46264</v>
+      <c r="A171" t="s">
+        <v>465</v>
       </c>
       <c r="B171" s="10" t="s">
         <v>18</v>
@@ -5937,8 +6046,8 @@
       <c r="G171" s="10"/>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A172" s="9">
-        <v>46264</v>
+      <c r="A172" t="s">
+        <v>465</v>
       </c>
       <c r="B172" s="10" t="s">
         <v>18</v>
@@ -5958,8 +6067,8 @@
       <c r="G172" s="10"/>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A173" s="9">
-        <v>46264</v>
+      <c r="A173" t="s">
+        <v>465</v>
       </c>
       <c r="B173" s="10" t="s">
         <v>18</v>
@@ -5982,8 +6091,8 @@
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A174" s="9">
-        <v>46264</v>
+      <c r="A174" t="s">
+        <v>465</v>
       </c>
       <c r="B174" s="10" t="s">
         <v>10</v>
@@ -6003,8 +6112,8 @@
       <c r="G174" s="10"/>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A175" s="9">
-        <v>46264</v>
+      <c r="A175" t="s">
+        <v>465</v>
       </c>
       <c r="B175" s="10" t="s">
         <v>10</v>
@@ -6024,8 +6133,8 @@
       <c r="G175" s="10"/>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A176" s="9">
-        <v>46264</v>
+      <c r="A176" t="s">
+        <v>465</v>
       </c>
       <c r="B176" s="10" t="s">
         <v>10</v>
@@ -6601,7 +6710,7 @@
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A200" s="9">
+      <c r="A200" s="8">
         <v>46270</v>
       </c>
       <c r="B200" s="10" t="s">
@@ -7019,8 +7128,8 @@
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A218" s="8">
-        <v>46274</v>
+      <c r="A218" t="s">
+        <v>282</v>
       </c>
       <c r="B218" t="s">
         <v>283</v>
@@ -7380,8 +7489,8 @@
       </c>
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A232" s="9">
-        <v>46275</v>
+      <c r="A232" t="s">
+        <v>462</v>
       </c>
       <c r="B232" s="10" t="s">
         <v>10</v>
@@ -7401,8 +7510,8 @@
       <c r="G232" s="10"/>
     </row>
     <row r="233" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A233" s="9">
-        <v>46275</v>
+      <c r="A233" t="s">
+        <v>462</v>
       </c>
       <c r="B233" s="10" t="s">
         <v>10</v>
@@ -7427,8 +7536,8 @@
       </c>
     </row>
     <row r="234" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A234" s="9">
-        <v>46275</v>
+      <c r="A234" t="s">
+        <v>462</v>
       </c>
       <c r="B234" s="10" t="s">
         <v>10</v>
@@ -7448,8 +7557,8 @@
       <c r="G234" s="10"/>
     </row>
     <row r="235" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A235" s="9">
-        <v>46275</v>
+      <c r="A235" t="s">
+        <v>462</v>
       </c>
       <c r="B235" s="10" t="s">
         <v>10</v>
@@ -7472,8 +7581,8 @@
       </c>
     </row>
     <row r="236" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A236" s="9">
-        <v>46275</v>
+      <c r="A236" t="s">
+        <v>462</v>
       </c>
       <c r="B236" s="10" t="s">
         <v>18</v>
@@ -7493,8 +7602,8 @@
       <c r="G236" s="10"/>
     </row>
     <row r="237" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A237" s="9">
-        <v>46275</v>
+      <c r="A237" t="s">
+        <v>462</v>
       </c>
       <c r="B237" s="10" t="s">
         <v>18</v>
@@ -7517,8 +7626,8 @@
       </c>
     </row>
     <row r="238" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A238" s="9">
-        <v>46275</v>
+      <c r="A238" t="s">
+        <v>462</v>
       </c>
       <c r="B238" s="10" t="s">
         <v>18</v>
@@ -7541,8 +7650,8 @@
       </c>
     </row>
     <row r="239" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A239" s="9">
-        <v>46275</v>
+      <c r="A239" t="s">
+        <v>462</v>
       </c>
       <c r="B239" s="10" t="s">
         <v>10</v>
@@ -7761,8 +7870,8 @@
       </c>
     </row>
     <row r="248" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A248" s="9">
-        <v>46277</v>
+      <c r="A248" t="s">
+        <v>460</v>
       </c>
       <c r="B248" s="10" t="s">
         <v>18</v>
@@ -7782,8 +7891,8 @@
       <c r="G248" s="10"/>
     </row>
     <row r="249" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A249" s="9">
-        <v>46277</v>
+      <c r="A249" t="s">
+        <v>460</v>
       </c>
       <c r="B249" s="10" t="s">
         <v>10</v>
@@ -7808,8 +7917,8 @@
       </c>
     </row>
     <row r="250" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A250" s="9">
-        <v>46277</v>
+      <c r="A250" t="s">
+        <v>460</v>
       </c>
       <c r="B250" s="10" t="s">
         <v>10</v>
@@ -7829,8 +7938,8 @@
       <c r="G250" s="10"/>
     </row>
     <row r="251" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A251" s="8">
-        <v>46278</v>
+      <c r="A251" t="s">
+        <v>461</v>
       </c>
       <c r="B251" s="10" t="s">
         <v>18</v>
@@ -7849,8 +7958,8 @@
       </c>
     </row>
     <row r="252" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A252" s="8">
-        <v>46278</v>
+      <c r="A252" t="s">
+        <v>461</v>
       </c>
       <c r="B252" s="10" t="s">
         <v>18</v>
@@ -7872,8 +7981,8 @@
       </c>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A253" s="8">
-        <v>46278</v>
+      <c r="A253" t="s">
+        <v>461</v>
       </c>
       <c r="B253" s="10" t="s">
         <v>18</v>
@@ -7892,8 +8001,8 @@
       </c>
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A254" s="8">
-        <v>46278</v>
+      <c r="A254" t="s">
+        <v>461</v>
       </c>
       <c r="B254" s="10" t="s">
         <v>10</v>
@@ -7915,8 +8024,8 @@
       </c>
     </row>
     <row r="255" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A255" s="8">
-        <v>46278</v>
+      <c r="A255" t="s">
+        <v>461</v>
       </c>
       <c r="B255" s="10" t="s">
         <v>10</v>
@@ -7935,8 +8044,8 @@
       </c>
     </row>
     <row r="256" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A256" s="8">
-        <v>46278</v>
+      <c r="A256" t="s">
+        <v>461</v>
       </c>
       <c r="B256" s="10" t="s">
         <v>10</v>
@@ -7955,8 +8064,8 @@
       </c>
     </row>
     <row r="257" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A257" s="8">
-        <v>46278</v>
+      <c r="A257" t="s">
+        <v>461</v>
       </c>
       <c r="B257" s="10" t="s">
         <v>10</v>
@@ -8629,8 +8738,8 @@
       </c>
     </row>
     <row r="285" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A285" s="9">
-        <v>46282</v>
+      <c r="A285" t="s">
+        <v>459</v>
       </c>
       <c r="B285" s="10" t="s">
         <v>283</v>
@@ -8650,8 +8759,8 @@
       <c r="G285" s="10"/>
     </row>
     <row r="286" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A286" s="9">
-        <v>46282</v>
+      <c r="A286" t="s">
+        <v>459</v>
       </c>
       <c r="B286" s="10" t="s">
         <v>283</v>
@@ -8671,8 +8780,8 @@
       <c r="G286" s="10"/>
     </row>
     <row r="287" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A287" s="9">
-        <v>46282</v>
+      <c r="A287" t="s">
+        <v>459</v>
       </c>
       <c r="B287" s="10" t="s">
         <v>283</v>
@@ -8692,8 +8801,8 @@
       <c r="G287" s="10"/>
     </row>
     <row r="288" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A288" s="9">
-        <v>46282</v>
+      <c r="A288" t="s">
+        <v>459</v>
       </c>
       <c r="B288" s="10" t="s">
         <v>283</v>
@@ -8713,8 +8822,8 @@
       <c r="G288" s="10"/>
     </row>
     <row r="289" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A289" s="9">
-        <v>46282</v>
+      <c r="A289" t="s">
+        <v>459</v>
       </c>
       <c r="B289" s="10" t="s">
         <v>283</v>
@@ -8734,8 +8843,8 @@
       <c r="G289" s="10"/>
     </row>
     <row r="290" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A290" s="9">
-        <v>46282</v>
+      <c r="A290" t="s">
+        <v>459</v>
       </c>
       <c r="B290" s="10" t="s">
         <v>283</v>
@@ -8758,8 +8867,8 @@
       </c>
     </row>
     <row r="291" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A291" s="9">
-        <v>46282</v>
+      <c r="A291" t="s">
+        <v>459</v>
       </c>
       <c r="B291" s="10" t="s">
         <v>18</v>
@@ -8784,8 +8893,8 @@
       </c>
     </row>
     <row r="292" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A292" s="9">
-        <v>46282</v>
+      <c r="A292" t="s">
+        <v>459</v>
       </c>
       <c r="B292" s="10" t="s">
         <v>18</v>
@@ -8810,8 +8919,8 @@
       </c>
     </row>
     <row r="293" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A293" s="9">
-        <v>46282</v>
+      <c r="A293" t="s">
+        <v>459</v>
       </c>
       <c r="B293" s="10" t="s">
         <v>18</v>
@@ -8833,8 +8942,8 @@
       </c>
     </row>
     <row r="294" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A294" s="9">
-        <v>46282</v>
+      <c r="A294" t="s">
+        <v>459</v>
       </c>
       <c r="B294" s="10" t="s">
         <v>18</v>
@@ -8854,8 +8963,8 @@
       <c r="G294" s="14"/>
     </row>
     <row r="295" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A295" s="9">
-        <v>46282</v>
+      <c r="A295" t="s">
+        <v>459</v>
       </c>
       <c r="B295" s="10" t="s">
         <v>18</v>
@@ -9113,8 +9222,8 @@
       </c>
     </row>
     <row r="306" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A306" s="9">
-        <v>46284</v>
+      <c r="A306" t="s">
+        <v>457</v>
       </c>
       <c r="B306" s="10" t="s">
         <v>18</v>
@@ -9134,8 +9243,8 @@
       <c r="G306" s="10"/>
     </row>
     <row r="307" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A307" s="9">
-        <v>46284</v>
+      <c r="A307" t="s">
+        <v>457</v>
       </c>
       <c r="B307" s="10" t="s">
         <v>18</v>
@@ -9155,8 +9264,8 @@
       <c r="G307" s="10"/>
     </row>
     <row r="308" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A308" s="9">
-        <v>46284</v>
+      <c r="A308" t="s">
+        <v>457</v>
       </c>
       <c r="B308" s="10" t="s">
         <v>18</v>
@@ -9181,8 +9290,8 @@
       </c>
     </row>
     <row r="309" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A309" s="9">
-        <v>46284</v>
+      <c r="A309" t="s">
+        <v>457</v>
       </c>
       <c r="B309" s="10" t="s">
         <v>18</v>
@@ -9202,8 +9311,8 @@
       <c r="G309" s="10"/>
     </row>
     <row r="310" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A310" s="9">
-        <v>46284</v>
+      <c r="A310" t="s">
+        <v>457</v>
       </c>
       <c r="B310" s="10" t="s">
         <v>10</v>
@@ -9223,8 +9332,8 @@
       <c r="G310" s="10"/>
     </row>
     <row r="311" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A311" s="9">
-        <v>46284</v>
+      <c r="A311" t="s">
+        <v>457</v>
       </c>
       <c r="B311" s="10" t="s">
         <v>10</v>
@@ -9244,8 +9353,8 @@
       <c r="G311" s="10"/>
     </row>
     <row r="312" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A312" s="9">
-        <v>46284</v>
+      <c r="A312" t="s">
+        <v>457</v>
       </c>
       <c r="B312" s="10" t="s">
         <v>375</v>
@@ -9268,8 +9377,8 @@
       </c>
     </row>
     <row r="313" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A313" s="9">
-        <v>46285</v>
+      <c r="A313" t="s">
+        <v>458</v>
       </c>
       <c r="B313" s="10" t="s">
         <v>375</v>
@@ -9289,8 +9398,8 @@
       <c r="G313" s="10"/>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A314" s="9">
-        <v>46285</v>
+      <c r="A314" t="s">
+        <v>458</v>
       </c>
       <c r="B314" s="10" t="s">
         <v>375</v>
@@ -9313,8 +9422,8 @@
       </c>
     </row>
     <row r="315" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A315" s="9">
-        <v>46285</v>
+      <c r="A315" t="s">
+        <v>458</v>
       </c>
       <c r="B315" s="10" t="s">
         <v>375</v>
@@ -9337,8 +9446,8 @@
       </c>
     </row>
     <row r="316" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A316" s="9">
-        <v>46285</v>
+      <c r="A316" t="s">
+        <v>458</v>
       </c>
       <c r="B316" s="10" t="s">
         <v>375</v>
@@ -9358,8 +9467,8 @@
       <c r="G316" s="10"/>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A317" s="9">
-        <v>46285</v>
+      <c r="A317" t="s">
+        <v>458</v>
       </c>
       <c r="B317" s="10" t="s">
         <v>375</v>
@@ -9379,8 +9488,8 @@
       <c r="G317" s="10"/>
     </row>
     <row r="318" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A318" s="9">
-        <v>46285</v>
+      <c r="A318" t="s">
+        <v>458</v>
       </c>
       <c r="B318" s="10" t="s">
         <v>375</v>
@@ -9403,8 +9512,8 @@
       </c>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A319" s="9">
-        <v>46285</v>
+      <c r="A319" t="s">
+        <v>458</v>
       </c>
       <c r="B319" s="10" t="s">
         <v>375</v>
@@ -9424,8 +9533,8 @@
       <c r="G319" s="10"/>
     </row>
     <row r="320" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A320" s="9">
-        <v>46285</v>
+      <c r="A320" t="s">
+        <v>458</v>
       </c>
       <c r="B320" s="10" t="s">
         <v>18</v>
@@ -9447,8 +9556,8 @@
       </c>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A321" s="9">
-        <v>46285</v>
+      <c r="A321" t="s">
+        <v>458</v>
       </c>
       <c r="B321" s="10" t="s">
         <v>18</v>
@@ -9468,8 +9577,8 @@
       <c r="G321" s="10"/>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A322" s="9">
-        <v>46285</v>
+      <c r="A322" t="s">
+        <v>458</v>
       </c>
       <c r="B322" s="10" t="s">
         <v>10</v>
@@ -10524,9 +10633,9 @@
         <v>227</v>
       </c>
     </row>
-    <row r="367" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A367" s="9">
-        <v>46289</v>
+    <row r="367" spans="1:8" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A367" t="s">
+        <v>422</v>
       </c>
       <c r="B367" s="10" t="s">
         <v>18</v>
@@ -10548,8 +10657,8 @@
       </c>
     </row>
     <row r="368" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A368" s="9">
-        <v>46289</v>
+      <c r="A368" t="s">
+        <v>422</v>
       </c>
       <c r="B368" s="10" t="s">
         <v>18</v>
@@ -10569,8 +10678,8 @@
       <c r="G368" s="10"/>
     </row>
     <row r="369" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A369" s="9">
-        <v>46289</v>
+      <c r="A369" t="s">
+        <v>422</v>
       </c>
       <c r="B369" s="10" t="s">
         <v>375</v>
@@ -10589,9 +10698,9 @@
       </c>
       <c r="G369" s="10"/>
     </row>
-    <row r="370" spans="1:8" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A370" s="9">
-        <v>46289</v>
+    <row r="370" spans="1:8" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A370" t="s">
+        <v>422</v>
       </c>
       <c r="B370" s="10" t="s">
         <v>10</v>
@@ -10613,9 +10722,543 @@
         <v>228</v>
       </c>
     </row>
+    <row r="371" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A371" t="s">
+        <v>454</v>
+      </c>
+      <c r="B371" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C371" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D371" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="E371" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F371" s="10"/>
+      <c r="G371" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="H371" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A372" t="s">
+        <v>454</v>
+      </c>
+      <c r="B372" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C372" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D372" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="E372" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F372" s="10">
+        <v>4.8099999999999996</v>
+      </c>
+      <c r="G372" s="10"/>
+    </row>
+    <row r="373" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A373" t="s">
+        <v>454</v>
+      </c>
+      <c r="B373" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C373" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D373" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E373" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F373" s="10">
+        <v>1.86</v>
+      </c>
+      <c r="G373" s="10"/>
+    </row>
+    <row r="374" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A374" t="s">
+        <v>454</v>
+      </c>
+      <c r="B374" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C374" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D374" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="E374" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F374" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="G374" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A375" t="s">
+        <v>454</v>
+      </c>
+      <c r="B375" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C375" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D375" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="E375" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F375" s="10">
+        <v>5.15</v>
+      </c>
+      <c r="G375" s="10"/>
+    </row>
+    <row r="376" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A376" t="s">
+        <v>454</v>
+      </c>
+      <c r="B376" s="10" t="s">
+        <v>375</v>
+      </c>
+      <c r="C376" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D376" s="10">
+        <v>2</v>
+      </c>
+      <c r="E376" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F376" s="10">
+        <v>4.49</v>
+      </c>
+      <c r="G376" s="10"/>
+    </row>
+    <row r="377" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A377" t="s">
+        <v>455</v>
+      </c>
+      <c r="B377" t="s">
+        <v>18</v>
+      </c>
+      <c r="C377" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D377" t="s">
+        <v>134</v>
+      </c>
+      <c r="E377" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F377" s="1">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="378" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A378" t="s">
+        <v>455</v>
+      </c>
+      <c r="B378" t="s">
+        <v>18</v>
+      </c>
+      <c r="C378" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D378" t="s">
+        <v>296</v>
+      </c>
+      <c r="E378" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G378" t="s">
+        <v>444</v>
+      </c>
+      <c r="H378" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="379" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A379" t="s">
+        <v>455</v>
+      </c>
+      <c r="B379" t="s">
+        <v>18</v>
+      </c>
+      <c r="C379" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D379" t="s">
+        <v>135</v>
+      </c>
+      <c r="E379" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F379" s="1">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="380" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A380" t="s">
+        <v>455</v>
+      </c>
+      <c r="B380" t="s">
+        <v>18</v>
+      </c>
+      <c r="C380" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D380" t="s">
+        <v>132</v>
+      </c>
+      <c r="E380" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F380" s="1">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="381" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A381" t="s">
+        <v>455</v>
+      </c>
+      <c r="B381" t="s">
+        <v>18</v>
+      </c>
+      <c r="C381" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D381" t="s">
+        <v>205</v>
+      </c>
+      <c r="E381" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G381" t="s">
+        <v>218</v>
+      </c>
+      <c r="H381" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="382" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A382" t="s">
+        <v>455</v>
+      </c>
+      <c r="B382" t="s">
+        <v>10</v>
+      </c>
+      <c r="C382" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D382" t="s">
+        <v>445</v>
+      </c>
+      <c r="E382" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G382" t="s">
+        <v>218</v>
+      </c>
+      <c r="H382" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="383" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A383" t="s">
+        <v>455</v>
+      </c>
+      <c r="B383" t="s">
+        <v>10</v>
+      </c>
+      <c r="C383" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D383" t="s">
+        <v>210</v>
+      </c>
+      <c r="E383" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F383" s="1">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="384" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A384" t="s">
+        <v>455</v>
+      </c>
+      <c r="B384" t="s">
+        <v>375</v>
+      </c>
+      <c r="C384" s="12" t="s">
+        <v>443</v>
+      </c>
+      <c r="D384" t="s">
+        <v>446</v>
+      </c>
+      <c r="E384" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F384" s="1">
+        <v>5.52</v>
+      </c>
+    </row>
+    <row r="385" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A385" t="s">
+        <v>456</v>
+      </c>
+      <c r="B385" t="s">
+        <v>375</v>
+      </c>
+      <c r="C385" s="15" t="s">
+        <v>453</v>
+      </c>
+      <c r="D385" t="s">
+        <v>447</v>
+      </c>
+      <c r="E385" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G385" t="s">
+        <v>200</v>
+      </c>
+      <c r="H385" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="386" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A386" t="s">
+        <v>456</v>
+      </c>
+      <c r="B386" t="s">
+        <v>10</v>
+      </c>
+      <c r="C386" s="15" t="s">
+        <v>453</v>
+      </c>
+      <c r="D386" t="s">
+        <v>448</v>
+      </c>
+      <c r="E386" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F386" s="1">
+        <v>3.36</v>
+      </c>
+      <c r="G386" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="387" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A387" t="s">
+        <v>456</v>
+      </c>
+      <c r="B387" t="s">
+        <v>18</v>
+      </c>
+      <c r="C387" s="15" t="s">
+        <v>453</v>
+      </c>
+      <c r="D387" t="s">
+        <v>174</v>
+      </c>
+      <c r="E387" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F387" s="1">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="388" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A388" t="s">
+        <v>456</v>
+      </c>
+      <c r="B388" t="s">
+        <v>18</v>
+      </c>
+      <c r="C388" s="15" t="s">
+        <v>453</v>
+      </c>
+      <c r="D388" t="s">
+        <v>139</v>
+      </c>
+      <c r="E388" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F388" s="1">
+        <v>3.61</v>
+      </c>
+      <c r="G388" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="389" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A389" t="s">
+        <v>456</v>
+      </c>
+      <c r="B389" t="s">
+        <v>18</v>
+      </c>
+      <c r="C389" s="15" t="s">
+        <v>453</v>
+      </c>
+      <c r="D389" t="s">
+        <v>451</v>
+      </c>
+      <c r="E389" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G389" t="s">
+        <v>452</v>
+      </c>
+      <c r="H389" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="390" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A390" t="s">
+        <v>467</v>
+      </c>
+      <c r="B390" t="s">
+        <v>18</v>
+      </c>
+      <c r="C390" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="D390" t="s">
+        <v>40</v>
+      </c>
+      <c r="E390" t="s">
+        <v>17</v>
+      </c>
+      <c r="F390" t="s">
+        <v>14</v>
+      </c>
+      <c r="G390" t="s">
+        <v>163</v>
+      </c>
+      <c r="H390" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="391" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A391" t="s">
+        <v>467</v>
+      </c>
+      <c r="B391" t="s">
+        <v>18</v>
+      </c>
+      <c r="C391" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="D391" t="s">
+        <v>96</v>
+      </c>
+      <c r="E391" t="s">
+        <v>17</v>
+      </c>
+      <c r="F391" t="s">
+        <v>14</v>
+      </c>
+      <c r="G391" t="s">
+        <v>163</v>
+      </c>
+      <c r="H391" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="392" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A392" t="s">
+        <v>467</v>
+      </c>
+      <c r="B392" t="s">
+        <v>10</v>
+      </c>
+      <c r="C392" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="D392" t="s">
+        <v>34</v>
+      </c>
+      <c r="E392" t="s">
+        <v>13</v>
+      </c>
+      <c r="F392" t="s">
+        <v>468</v>
+      </c>
+      <c r="G392" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="393" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A393" t="s">
+        <v>467</v>
+      </c>
+      <c r="B393" t="s">
+        <v>18</v>
+      </c>
+      <c r="C393" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="D393" t="s">
+        <v>40</v>
+      </c>
+      <c r="E393" t="s">
+        <v>13</v>
+      </c>
+      <c r="F393" t="s">
+        <v>470</v>
+      </c>
+      <c r="G393" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="394" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A394" t="s">
+        <v>467</v>
+      </c>
+      <c r="B394" t="s">
+        <v>18</v>
+      </c>
+      <c r="C394" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="D394" t="s">
+        <v>96</v>
+      </c>
+      <c r="E394" t="s">
+        <v>13</v>
+      </c>
+      <c r="F394" t="s">
+        <v>472</v>
+      </c>
+      <c r="G394" t="s">
+        <v>473</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A2:E3 A12:E18 A10:E11 A26:E27 A1:E1 A5:E7 A4:E4 G4 A9:E9 A8:E8 G8 A20:E24 A19:E19 G19 G2:G3 G12:G18 G1 G5:G7 G9 G20:G25 A25:D25" numberStoredAsText="1"/>
   </ignoredErrors>
@@ -10648,7 +11291,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{240BDDD7-65A5-4F9A-8645-E6E255B43C11}">
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.75" customWidth="1"/>
@@ -13148,6 +13791,259 @@
       </c>
       <c r="G110" s="1">
         <v>1.27</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A111" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C111" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D111" s="1">
+        <v>4</v>
+      </c>
+      <c r="E111" s="1">
+        <v>3</v>
+      </c>
+      <c r="F111" s="1">
+        <v>1</v>
+      </c>
+      <c r="G111" s="1">
+        <v>15.94</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A112" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B112" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C112" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D112" s="1">
+        <v>1</v>
+      </c>
+      <c r="E112" s="1">
+        <v>1</v>
+      </c>
+      <c r="F112" s="1">
+        <v>0</v>
+      </c>
+      <c r="G112" s="1">
+        <v>7.24</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A113" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="C113" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D113" s="1">
+        <v>1</v>
+      </c>
+      <c r="E113" s="1">
+        <v>1</v>
+      </c>
+      <c r="F113" s="1">
+        <v>0</v>
+      </c>
+      <c r="G113" s="1">
+        <v>5.58</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A114" s="8">
+        <v>46291</v>
+      </c>
+      <c r="B114" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C114" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D114" s="1">
+        <v>5</v>
+      </c>
+      <c r="E114" s="1">
+        <v>3</v>
+      </c>
+      <c r="F114" s="1">
+        <v>2</v>
+      </c>
+      <c r="G114" s="1">
+        <v>22.48</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A115" s="8">
+        <v>46291</v>
+      </c>
+      <c r="B115" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C115" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D115" s="1">
+        <v>2</v>
+      </c>
+      <c r="E115" s="1">
+        <v>1</v>
+      </c>
+      <c r="F115" s="1">
+        <v>1</v>
+      </c>
+      <c r="G115" s="1">
+        <v>7.42</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A116" s="8">
+        <v>46291</v>
+      </c>
+      <c r="B116" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="C116" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="D116" s="1">
+        <v>1</v>
+      </c>
+      <c r="E116" s="1">
+        <v>1</v>
+      </c>
+      <c r="F116" s="1">
+        <v>0</v>
+      </c>
+      <c r="G116" s="1">
+        <v>7.18</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A117" s="8">
+        <v>46292</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="C117" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="D117" s="1">
+        <v>1</v>
+      </c>
+      <c r="E117" s="1">
+        <v>0</v>
+      </c>
+      <c r="F117" s="1">
+        <v>1</v>
+      </c>
+      <c r="G117" s="1">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A118" s="8">
+        <v>46292</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C118" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="D118" s="1">
+        <v>1</v>
+      </c>
+      <c r="E118" s="1">
+        <v>1</v>
+      </c>
+      <c r="F118" s="1">
+        <v>0</v>
+      </c>
+      <c r="G118" s="1">
+        <v>7.35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A119" s="8">
+        <v>46292</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C119" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="D119" s="1">
+        <v>3</v>
+      </c>
+      <c r="E119" s="1">
+        <v>2</v>
+      </c>
+      <c r="F119" s="1">
+        <v>1</v>
+      </c>
+      <c r="G119" s="1">
+        <v>9.2799999999999994</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>467</v>
+      </c>
+      <c r="B120" t="s">
+        <v>18</v>
+      </c>
+      <c r="C120" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="D120">
+        <v>4</v>
+      </c>
+      <c r="E120">
+        <v>2</v>
+      </c>
+      <c r="F120">
+        <v>2</v>
+      </c>
+      <c r="G120" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>467</v>
+      </c>
+      <c r="B121" t="s">
+        <v>10</v>
+      </c>
+      <c r="C121" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="D121">
+        <v>1</v>
+      </c>
+      <c r="E121">
+        <v>1</v>
+      </c>
+      <c r="F121">
+        <v>0</v>
+      </c>
+      <c r="G121" t="s">
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -13213,7 +14109,7 @@
       </c>
       <c r="B7" s="3">
         <f>AVERAGEIF(Patient_Log!F2:F997,"&lt;&gt;0")</f>
-        <v>3.9786394557823122</v>
+        <v>3.8874999999999984</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -13225,7 +14121,7 @@
       </c>
       <c r="B9" s="1">
         <f>SUM(Unit_Log!E2:E1000)</f>
-        <v>305</v>
+        <v>321</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
changed the time from ISOString (which is hardcoded for UTC) to this time zone so it stops giving output for the next day after a certain time
</commit_message>
<xml_diff>
--- a/Select_Menu_Patient_Log.xlsx
+++ b/Select_Menu_Patient_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dvagov-my.sharepoint.com/personal/crystal_alvarez_va_gov/Documents/Desktop/Select Menu/VSCode/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1215" documentId="13_ncr:1_{9CEB82FD-F55C-4572-8711-23C7E1DF9E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D4ECE6F-3EB2-471E-8E6F-D2888B5FF305}"/>
+  <xr:revisionPtr revIDLastSave="1511" documentId="13_ncr:1_{9CEB82FD-F55C-4572-8711-23C7E1DF9E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59C4F8F8-3F53-4CA0-8123-4B2A90A1A9E0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient_Log" sheetId="1" r:id="rId1"/>
@@ -250,7 +250,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3476" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4370" uniqueCount="500">
   <si>
     <t>Date</t>
   </si>
@@ -1411,6 +1411,345 @@
   </si>
   <si>
     <t>ICU-7</t>
+  </si>
+  <si>
+    <t>with provider</t>
+  </si>
+  <si>
+    <t>profile locked</t>
+  </si>
+  <si>
+    <t>modified LDAs</t>
+  </si>
+  <si>
+    <t>patient is very particular lots of changes</t>
+  </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
+    <t>9.13</t>
+  </si>
+  <si>
+    <t>extra few minutes for survey</t>
+  </si>
+  <si>
+    <t>discharging. did survey though. mentioned giving toothpicks would be nice.</t>
+  </si>
+  <si>
+    <t>change timer to add 4 minutes</t>
+  </si>
+  <si>
+    <t>5.59</t>
+  </si>
+  <si>
+    <t>2.26</t>
+  </si>
+  <si>
+    <t>2.79</t>
+  </si>
+  <si>
+    <t>9.78</t>
+  </si>
+  <si>
+    <t>tray missing items</t>
+  </si>
+  <si>
+    <t>31.99</t>
+  </si>
+  <si>
+    <t>25.24</t>
+  </si>
+  <si>
+    <t>discharge</t>
+  </si>
+  <si>
+    <t>2c16</t>
+  </si>
+  <si>
+    <t>pt w/provider</t>
+  </si>
+  <si>
+    <t>NO MILK</t>
+  </si>
+  <si>
+    <t>Patient is hard of hearing.</t>
+  </si>
+  <si>
+    <t>Patient is nonresponsive</t>
+  </si>
+  <si>
+    <t>Patient is sleeping</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>PATIENT WAS NOT FEELING WELL I CHOSE THE MEALS FOR HIM</t>
+  </si>
+  <si>
+    <t>NPO</t>
+  </si>
+  <si>
+    <t>ICU-6</t>
+  </si>
+  <si>
+    <t>patient wants strawberry ice cream everyday</t>
+  </si>
+  <si>
+    <t>pt eating lunch, he wants me to come back after.</t>
+  </si>
+  <si>
+    <t>3A02</t>
+  </si>
+  <si>
+    <t>pt wants diet cola w/ lunch or dinner</t>
+  </si>
+  <si>
+    <t>pt is not available so i went w/ marci to check expiration dates in nourishment rooms</t>
+  </si>
+  <si>
+    <t>w provider</t>
+  </si>
+  <si>
+    <t>provider came in at end. pt is upset bc "worlds worst breakfast" will come back later to finish for lunch and dinner for tm.</t>
+  </si>
+  <si>
+    <t>8:30 AM</t>
+  </si>
+  <si>
+    <t>C 16</t>
+  </si>
+  <si>
+    <t>pt with nurse</t>
+  </si>
+  <si>
+    <t>pt is on hospice and is a little confused</t>
+  </si>
+  <si>
+    <t>hospice pt, expressed some difficulty with hospice menu and kept talking</t>
+  </si>
+  <si>
+    <t>pt likes broccoli</t>
+  </si>
+  <si>
+    <t>2B13</t>
+  </si>
+  <si>
+    <t>2B17</t>
+  </si>
+  <si>
+    <t>pt discharging tmw</t>
+  </si>
+  <si>
+    <t>2B26</t>
+  </si>
+  <si>
+    <t>pt is sleeping, did not eat his dinner tray and i cannot wake him</t>
+  </si>
+  <si>
+    <t>3A05</t>
+  </si>
+  <si>
+    <t>pt needs dietician consult</t>
+  </si>
+  <si>
+    <t>pt discharging in a few moments</t>
+  </si>
+  <si>
+    <t>3A07</t>
+  </si>
+  <si>
+    <t>3A19</t>
+  </si>
+  <si>
+    <t>pt wants chef salad</t>
+  </si>
+  <si>
+    <t>3A26</t>
+  </si>
+  <si>
+    <t>3A29</t>
+  </si>
+  <si>
+    <t>pt requests not at this time</t>
+  </si>
+  <si>
+    <t>2C16</t>
+  </si>
+  <si>
+    <t>6:00 PM</t>
+  </si>
+  <si>
+    <t>pt in pain. didn't really want to talk but let me finish his meals</t>
+  </si>
+  <si>
+    <t>pt has a lot of difficulty hearing. had to speak loudly. he was very eager about the menu!</t>
+  </si>
+  <si>
+    <t>pt just had difficulty speaking and spoke slowly. said he "supports what we're doing 100%" (referring to select menu)</t>
+  </si>
+  <si>
+    <t>took long deciding on items</t>
+  </si>
+  <si>
+    <t>pt in pain but willing to go over his meals</t>
+  </si>
+  <si>
+    <t>room stripped. possible DC</t>
+  </si>
+  <si>
+    <t>provider needed him for a procedure so we only did his dinner tray for tonight</t>
+  </si>
+  <si>
+    <t>PATIENT WOULD LIKE LARGE PROTIONS FOR MEALS I WILL NOTIFY STAFF</t>
+  </si>
+  <si>
+    <t>NO COFFEE</t>
+  </si>
+  <si>
+    <t>DOES NOT EAT CHICKEN OR BEEF</t>
+  </si>
+  <si>
+    <t>DISLIKES RAW ONION</t>
+  </si>
+  <si>
+    <t>PATIENT SLEEP</t>
+  </si>
+  <si>
+    <t>B24</t>
+  </si>
+  <si>
+    <t>PATIENT IS SLEEPING</t>
+  </si>
+  <si>
+    <t>SLEEP HOSPICE PATIENT</t>
+  </si>
+  <si>
+    <t>PATIENT SAYS IT'S TOO MUCH FOOD. I EXPLAINED THE PORTION SIZES TO HIM AND STILL THINKS IT'S TOO MUCH.</t>
+  </si>
+  <si>
+    <t>DISLIKES FISH.  ENTERED IN DISLIKES</t>
+  </si>
+  <si>
+    <t>PATIENT IS FREQUENTLY SLEEP</t>
+  </si>
+  <si>
+    <t>PATIENT SAYS HE WILL EAT ANYTHING AND HAS NO PREFERENCES</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>pt discharged. room being flipped</t>
+  </si>
+  <si>
+    <t>7.96</t>
+  </si>
+  <si>
+    <t>pt was slightly incoherent. had difficulty understanding him (mumbling) but read the menu to him and that was fine.</t>
+  </si>
+  <si>
+    <t>3.06</t>
+  </si>
+  <si>
+    <t>3.65</t>
+  </si>
+  <si>
+    <t>w/ provider and asleep</t>
+  </si>
+  <si>
+    <t>5.05</t>
+  </si>
+  <si>
+    <t>8.84</t>
+  </si>
+  <si>
+    <t>prefers smaller trays w/ less food on them</t>
+  </si>
+  <si>
+    <t>2.92</t>
+  </si>
+  <si>
+    <t>still w/ provider</t>
+  </si>
+  <si>
+    <t>26.40</t>
+  </si>
+  <si>
+    <t>2.61</t>
+  </si>
+  <si>
+    <t>30.68</t>
+  </si>
+  <si>
+    <t>patient is discharging tmw</t>
+  </si>
+  <si>
+    <t>pt getting an IV</t>
+  </si>
+  <si>
+    <t>3A24</t>
+  </si>
+  <si>
+    <t>pt with physical therapist</t>
+  </si>
+  <si>
+    <t>pt wants diet sprite and no coffee on trays</t>
+  </si>
+  <si>
+    <t>pt is asking for sandwiches between meals, as was promised to him.</t>
+  </si>
+  <si>
+    <t>pt is getting discharged at noon</t>
+  </si>
+  <si>
+    <t>pt being prepped for a procedure not a good time</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>pt would like to try blue cheese dressing</t>
+  </si>
+  <si>
+    <t>pt wants vanilla ensure</t>
+  </si>
+  <si>
+    <t>pt dislikes fish</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>12.59</t>
+  </si>
+  <si>
+    <t>2.73</t>
+  </si>
+  <si>
+    <t>20.60</t>
+  </si>
+  <si>
+    <t>pt mentioned allergies. has not had RD consult. We reviewed trays and recipes carefully, while considering allergies</t>
+  </si>
+  <si>
+    <t>5.26</t>
+  </si>
+  <si>
+    <t>8.03</t>
+  </si>
+  <si>
+    <t>pt disoriented w/ difficulty focusing. Resorted to chef selections and did not make changes to trays for tomorrow</t>
+  </si>
+  <si>
+    <t>pt. discharging</t>
+  </si>
+  <si>
+    <t>62.14</t>
+  </si>
+  <si>
+    <t>9.67</t>
   </si>
 </sst>
 </file>
@@ -1532,8 +1871,8 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1891,7 +2230,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H494"/>
+  <dimension ref="A1:H643"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -11803,7 +12142,7 @@
       <c r="E438" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F438" s="17">
+      <c r="F438" s="1">
         <v>14.49</v>
       </c>
       <c r="G438" t="s">
@@ -11826,7 +12165,7 @@
       <c r="E439" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F439" s="17">
+      <c r="F439" s="1">
         <v>4.72</v>
       </c>
       <c r="G439" t="s">
@@ -11849,7 +12188,7 @@
       <c r="E440" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F440" s="17">
+      <c r="F440" s="1">
         <v>2.74</v>
       </c>
       <c r="G440" t="s">
@@ -11893,7 +12232,7 @@
       <c r="E442" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F442" s="17">
+      <c r="F442" s="1">
         <v>6.34</v>
       </c>
       <c r="G442" t="s">
@@ -11916,7 +12255,7 @@
       <c r="E443" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F443" s="17">
+      <c r="F443" s="1">
         <v>11.44</v>
       </c>
       <c r="G443" t="s">
@@ -13022,6 +13361,3351 @@
       </c>
       <c r="F494" s="1">
         <v>1.04</v>
+      </c>
+    </row>
+    <row r="495" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A495" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B495" t="s">
+        <v>10</v>
+      </c>
+      <c r="C495" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D495" s="1">
+        <v>2</v>
+      </c>
+      <c r="E495" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G495" s="14" t="s">
+        <v>387</v>
+      </c>
+      <c r="H495" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="496" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A496" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B496" t="s">
+        <v>10</v>
+      </c>
+      <c r="C496" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D496" s="1">
+        <v>4</v>
+      </c>
+      <c r="E496" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F496" s="1">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="497" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A497" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B497" t="s">
+        <v>10</v>
+      </c>
+      <c r="C497" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D497" s="1">
+        <v>2</v>
+      </c>
+      <c r="E497" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G497" s="14" t="s">
+        <v>388</v>
+      </c>
+      <c r="H497" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="498" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A498" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B498" t="s">
+        <v>10</v>
+      </c>
+      <c r="C498" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D498" s="1">
+        <v>5</v>
+      </c>
+      <c r="E498" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F498" s="1">
+        <v>4.09</v>
+      </c>
+    </row>
+    <row r="499" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A499" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B499" t="s">
+        <v>18</v>
+      </c>
+      <c r="C499" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D499" s="1">
+        <v>20</v>
+      </c>
+      <c r="E499" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F499" s="1">
+        <v>4.1900000000000004</v>
+      </c>
+      <c r="G499" s="14" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="500" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A500" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B500" t="s">
+        <v>18</v>
+      </c>
+      <c r="C500" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D500" s="1">
+        <v>26</v>
+      </c>
+      <c r="E500" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F500" s="1">
+        <v>2.5099999999999998</v>
+      </c>
+    </row>
+    <row r="501" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A501" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B501" t="s">
+        <v>18</v>
+      </c>
+      <c r="C501" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D501" s="1">
+        <v>17</v>
+      </c>
+      <c r="E501" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F501" s="1">
+        <v>21.38</v>
+      </c>
+      <c r="G501" s="14" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="502" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A502" t="s">
+        <v>391</v>
+      </c>
+      <c r="B502" t="s">
+        <v>10</v>
+      </c>
+      <c r="C502" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D502" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E502" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F502" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="G502" s="14" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="503" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A503" t="s">
+        <v>391</v>
+      </c>
+      <c r="B503" t="s">
+        <v>10</v>
+      </c>
+      <c r="C503" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D503" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E503" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F503" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G503" s="14" t="s">
+        <v>394</v>
+      </c>
+      <c r="H503" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="504" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A504" t="s">
+        <v>391</v>
+      </c>
+      <c r="B504" t="s">
+        <v>10</v>
+      </c>
+      <c r="C504" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D504" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E504" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F504" s="1">
+        <v>6.86</v>
+      </c>
+      <c r="G504" s="14" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="505" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A505" t="s">
+        <v>391</v>
+      </c>
+      <c r="B505" t="s">
+        <v>10</v>
+      </c>
+      <c r="C505" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D505" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E505" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F505" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G505" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="H505" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="506" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A506" t="s">
+        <v>391</v>
+      </c>
+      <c r="B506" t="s">
+        <v>18</v>
+      </c>
+      <c r="C506" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D506" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E506" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F506" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="G506" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="507" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A507" t="s">
+        <v>391</v>
+      </c>
+      <c r="B507" t="s">
+        <v>18</v>
+      </c>
+      <c r="C507" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D507" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E507" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F507" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="G507" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="508" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A508" t="s">
+        <v>391</v>
+      </c>
+      <c r="B508" t="s">
+        <v>18</v>
+      </c>
+      <c r="C508" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D508" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E508" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F508" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="G508" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="509" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A509" t="s">
+        <v>391</v>
+      </c>
+      <c r="B509" t="s">
+        <v>18</v>
+      </c>
+      <c r="C509" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D509" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E509" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F509" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="G509" s="14" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="510" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A510" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B510" t="s">
+        <v>18</v>
+      </c>
+      <c r="C510" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D510" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E510" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F510" s="1">
+        <v>3.38</v>
+      </c>
+      <c r="G510"/>
+    </row>
+    <row r="511" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A511" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B511" t="s">
+        <v>18</v>
+      </c>
+      <c r="C511" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D511" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E511" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G511" t="s">
+        <v>403</v>
+      </c>
+      <c r="H511" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="512" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A512" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B512" t="s">
+        <v>18</v>
+      </c>
+      <c r="C512" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D512" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E512" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G512" t="s">
+        <v>141</v>
+      </c>
+      <c r="H512" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="513" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A513" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B513" t="s">
+        <v>18</v>
+      </c>
+      <c r="C513" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D513" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E513" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F513" s="1">
+        <v>4.37</v>
+      </c>
+      <c r="G513"/>
+    </row>
+    <row r="514" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A514" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B514" t="s">
+        <v>18</v>
+      </c>
+      <c r="C514" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D514" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E514" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G514" t="s">
+        <v>405</v>
+      </c>
+      <c r="H514" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="515" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A515" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B515" t="s">
+        <v>18</v>
+      </c>
+      <c r="C515" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D515" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E515" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F515" s="1">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="516" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A516" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B516" t="s">
+        <v>18</v>
+      </c>
+      <c r="C516" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D516" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E516" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F516" s="1">
+        <v>2.66</v>
+      </c>
+      <c r="G516" s="14" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="517" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A517" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B517" t="s">
+        <v>10</v>
+      </c>
+      <c r="C517" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D517" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E517" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F517" s="1">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="518" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A518" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B518" t="s">
+        <v>10</v>
+      </c>
+      <c r="C518" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D518" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E518" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F518" s="1">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="G518" s="14" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="519" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A519" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B519" t="s">
+        <v>10</v>
+      </c>
+      <c r="C519" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D519" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="E519" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G519" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="H519" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="520" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A520" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B520" t="s">
+        <v>10</v>
+      </c>
+      <c r="C520" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D520" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="E520" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F520" s="1">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="521" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A521" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B521" t="s">
+        <v>271</v>
+      </c>
+      <c r="C521" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D521" s="1">
+        <v>1</v>
+      </c>
+      <c r="E521" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F521" s="1">
+        <v>2.87</v>
+      </c>
+    </row>
+    <row r="522" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A522" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B522" t="s">
+        <v>271</v>
+      </c>
+      <c r="C522" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D522" s="1">
+        <v>6</v>
+      </c>
+      <c r="E522" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G522" s="14" t="s">
+        <v>409</v>
+      </c>
+      <c r="H522" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="523" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A523" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B523" t="s">
+        <v>18</v>
+      </c>
+      <c r="C523" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D523" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="E523" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F523" s="1">
+        <v>4.66</v>
+      </c>
+    </row>
+    <row r="524" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A524" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B524" t="s">
+        <v>18</v>
+      </c>
+      <c r="C524" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D524" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E524" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F524" s="1">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="525" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A525" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B525" t="s">
+        <v>18</v>
+      </c>
+      <c r="C525" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D525" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E525" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F525" s="1">
+        <v>1.59</v>
+      </c>
+    </row>
+    <row r="526" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A526" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B526" t="s">
+        <v>18</v>
+      </c>
+      <c r="C526" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D526" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E526" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G526" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="H526" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="527" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A527" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B527" t="s">
+        <v>10</v>
+      </c>
+      <c r="C527" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D527" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E527" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F527" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="G527" s="14" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="528" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A528" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B528" t="s">
+        <v>10</v>
+      </c>
+      <c r="C528" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D528" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E528" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F528" s="1">
+        <v>4.18</v>
+      </c>
+    </row>
+    <row r="529" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A529" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B529" t="s">
+        <v>10</v>
+      </c>
+      <c r="C529" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D529" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="E529" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F529" s="1">
+        <v>0.27</v>
+      </c>
+      <c r="G529" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="H529" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="530" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A530" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B530" t="s">
+        <v>271</v>
+      </c>
+      <c r="C530" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D530" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E530" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F530" s="1">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="531" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A531" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B531" t="s">
+        <v>10</v>
+      </c>
+      <c r="C531" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D531" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="E531" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F531" s="1">
+        <v>4.5599999999999996</v>
+      </c>
+      <c r="G531" s="14" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="532" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A532" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B532" t="s">
+        <v>18</v>
+      </c>
+      <c r="C532" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D532" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E532" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F532" s="1">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="533" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A533" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B533" t="s">
+        <v>18</v>
+      </c>
+      <c r="C533" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D533" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E533" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G533" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="H533" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="534" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A534" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B534" t="s">
+        <v>18</v>
+      </c>
+      <c r="C534" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D534" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E534" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G534" s="14" t="s">
+        <v>415</v>
+      </c>
+      <c r="H534" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="535" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A535" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B535" t="s">
+        <v>10</v>
+      </c>
+      <c r="C535" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D535" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="E535" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F535" s="1">
+        <v>4.42</v>
+      </c>
+      <c r="G535" s="14" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="536" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A536" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B536" t="s">
+        <v>18</v>
+      </c>
+      <c r="C536" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D536" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E536" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G536" s="14" t="s">
+        <v>418</v>
+      </c>
+      <c r="H536" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="537" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A537" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B537" t="s">
+        <v>18</v>
+      </c>
+      <c r="C537" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D537" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E537" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F537" s="1">
+        <v>8.5399999999999991</v>
+      </c>
+    </row>
+    <row r="538" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A538" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B538" t="s">
+        <v>18</v>
+      </c>
+      <c r="C538" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D538" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E538" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F538" s="1">
+        <v>7.97</v>
+      </c>
+    </row>
+    <row r="539" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A539" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B539" t="s">
+        <v>18</v>
+      </c>
+      <c r="C539" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D539" s="1">
+        <v>11</v>
+      </c>
+      <c r="E539" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G539" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="H539" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="540" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A540" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B540" t="s">
+        <v>18</v>
+      </c>
+      <c r="C540" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D540" s="1">
+        <v>13</v>
+      </c>
+      <c r="E540" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F540" s="1">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="541" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A541" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B541" t="s">
+        <v>18</v>
+      </c>
+      <c r="C541" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D541" s="1">
+        <v>16</v>
+      </c>
+      <c r="E541" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G541" s="14" t="s">
+        <v>375</v>
+      </c>
+      <c r="H541" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="542" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A542" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B542" t="s">
+        <v>10</v>
+      </c>
+      <c r="C542" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D542" s="1">
+        <v>17</v>
+      </c>
+      <c r="E542" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F542" s="1">
+        <v>5.62</v>
+      </c>
+    </row>
+    <row r="543" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A543" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B543" t="s">
+        <v>10</v>
+      </c>
+      <c r="C543" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D543" s="1">
+        <v>21</v>
+      </c>
+      <c r="E543" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F543" s="1">
+        <v>8.02</v>
+      </c>
+      <c r="G543" s="14" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="544" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A544" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B544" t="s">
+        <v>10</v>
+      </c>
+      <c r="C544" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D544" s="1">
+        <v>6</v>
+      </c>
+      <c r="E544" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F544" s="1">
+        <v>4.53</v>
+      </c>
+    </row>
+    <row r="545" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A545" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B545" t="s">
+        <v>10</v>
+      </c>
+      <c r="C545" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D545" s="1">
+        <v>2</v>
+      </c>
+      <c r="E545" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F545" s="1">
+        <v>5.55</v>
+      </c>
+    </row>
+    <row r="546" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A546" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B546" t="s">
+        <v>18</v>
+      </c>
+      <c r="C546" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D546" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="E546" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G546" s="14" t="s">
+        <v>423</v>
+      </c>
+      <c r="H546" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="547" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A547" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B547" t="s">
+        <v>18</v>
+      </c>
+      <c r="C547" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D547" s="1">
+        <v>17</v>
+      </c>
+      <c r="E547" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G547" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="H547" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="548" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A548" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B548" t="s">
+        <v>18</v>
+      </c>
+      <c r="C548" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D548" s="1">
+        <v>26</v>
+      </c>
+      <c r="E548" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F548" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="G548" s="14" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="549" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A549" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B549" t="s">
+        <v>18</v>
+      </c>
+      <c r="C549" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D549" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="E549" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F549" s="1">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="G549" s="14" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="550" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A550" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B550" t="s">
+        <v>18</v>
+      </c>
+      <c r="C550" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D550" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="E550" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F550" s="1">
+        <v>2.82</v>
+      </c>
+      <c r="G550" s="14" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="551" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A551" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B551" t="s">
+        <v>18</v>
+      </c>
+      <c r="C551" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D551" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="E551" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G551" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="H551" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="552" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A552" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B552" t="s">
+        <v>18</v>
+      </c>
+      <c r="C552" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D552" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="E552" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F552" s="1">
+        <v>1.51</v>
+      </c>
+      <c r="G552" s="14" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="553" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A553" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B553" t="s">
+        <v>18</v>
+      </c>
+      <c r="C553" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D553" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="E553" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G553" s="14" t="s">
+        <v>431</v>
+      </c>
+      <c r="H553" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="554" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A554" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B554" t="s">
+        <v>10</v>
+      </c>
+      <c r="C554" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D554" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="E554" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G554" s="14" t="s">
+        <v>433</v>
+      </c>
+      <c r="H554" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="555" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A555" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B555" t="s">
+        <v>10</v>
+      </c>
+      <c r="C555" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D555" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="E555" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G555" s="14" t="s">
+        <v>434</v>
+      </c>
+      <c r="H555" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="556" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A556" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B556" t="s">
+        <v>10</v>
+      </c>
+      <c r="C556" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D556" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="E556" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F556" s="1">
+        <v>2.41</v>
+      </c>
+    </row>
+    <row r="557" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A557" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B557" t="s">
+        <v>10</v>
+      </c>
+      <c r="C557" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D557" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="E557" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F557" s="1">
+        <v>7.39</v>
+      </c>
+      <c r="G557" s="14" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="558" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A558" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B558" t="s">
+        <v>10</v>
+      </c>
+      <c r="C558" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D558" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="E558" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F558" s="1">
+        <v>2.5499999999999998</v>
+      </c>
+    </row>
+    <row r="559" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A559" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B559" t="s">
+        <v>10</v>
+      </c>
+      <c r="C559" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D559" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="E559" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F559" s="1">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="560" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A560" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B560" t="s">
+        <v>10</v>
+      </c>
+      <c r="C560" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D560" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="E560" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G560" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="H560" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="561" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A561" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B561" t="s">
+        <v>18</v>
+      </c>
+      <c r="C561" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D561" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="E561" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F561" s="1">
+        <v>21.24</v>
+      </c>
+    </row>
+    <row r="562" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A562" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B562" t="s">
+        <v>10</v>
+      </c>
+      <c r="C562" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D562" s="1">
+        <v>2</v>
+      </c>
+      <c r="E562" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F562" s="1">
+        <v>7.17</v>
+      </c>
+      <c r="G562" s="14" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="563" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A563" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B563" t="s">
+        <v>10</v>
+      </c>
+      <c r="C563" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D563" s="1">
+        <v>7</v>
+      </c>
+      <c r="E563" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G563" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H563" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="564" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A564" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B564" t="s">
+        <v>10</v>
+      </c>
+      <c r="C564" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D564" s="1">
+        <v>19</v>
+      </c>
+      <c r="E564" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G564" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="H564" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="565" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A565" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B565" t="s">
+        <v>10</v>
+      </c>
+      <c r="C565" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D565" s="1">
+        <v>29</v>
+      </c>
+      <c r="E565" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F565" s="1">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="566" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A566" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B566" t="s">
+        <v>10</v>
+      </c>
+      <c r="C566" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D566" s="1">
+        <v>6</v>
+      </c>
+      <c r="E566" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G566" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H566" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="567" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A567" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B567" t="s">
+        <v>18</v>
+      </c>
+      <c r="C567" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D567" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E567" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F567" s="1">
+        <v>6.46</v>
+      </c>
+    </row>
+    <row r="568" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A568" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B568" t="s">
+        <v>18</v>
+      </c>
+      <c r="C568" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D568" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="E568" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F568" s="1">
+        <v>17.59</v>
+      </c>
+      <c r="G568" s="14" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="569" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A569" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B569" t="s">
+        <v>18</v>
+      </c>
+      <c r="C569" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D569" s="1">
+        <v>26</v>
+      </c>
+      <c r="E569" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F569" s="1">
+        <v>3.21</v>
+      </c>
+      <c r="G569" s="14" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="570" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A570" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B570" t="s">
+        <v>10</v>
+      </c>
+      <c r="C570" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D570" s="1">
+        <v>6</v>
+      </c>
+      <c r="E570" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G570" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H570" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="571" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A571" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B571" t="s">
+        <v>10</v>
+      </c>
+      <c r="C571" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D571" s="1">
+        <v>7</v>
+      </c>
+      <c r="E571" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G571" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H571" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="572" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A572" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B572" t="s">
+        <v>10</v>
+      </c>
+      <c r="C572" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D572" s="1">
+        <v>6</v>
+      </c>
+      <c r="E572" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F572" s="1">
+        <v>20.350000000000001</v>
+      </c>
+      <c r="G572" s="14" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="573" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A573" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B573" t="s">
+        <v>10</v>
+      </c>
+      <c r="C573" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D573" s="1">
+        <v>7</v>
+      </c>
+      <c r="E573" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G573" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H573" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="574" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A574" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B574" t="s">
+        <v>18</v>
+      </c>
+      <c r="C574" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D574" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="E574" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F574" s="1">
+        <v>12.82</v>
+      </c>
+    </row>
+    <row r="575" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A575" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B575" t="s">
+        <v>18</v>
+      </c>
+      <c r="C575" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D575" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="E575" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F575" s="1">
+        <v>15.45</v>
+      </c>
+    </row>
+    <row r="576" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A576" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B576" t="s">
+        <v>18</v>
+      </c>
+      <c r="C576" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D576" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E576" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F576" s="1">
+        <v>2.0099999999999998</v>
+      </c>
+    </row>
+    <row r="577" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A577" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B577" t="s">
+        <v>18</v>
+      </c>
+      <c r="C577" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D577" s="1">
+        <v>28</v>
+      </c>
+      <c r="E577" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G577" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="H577" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="578" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A578" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B578" t="s">
+        <v>10</v>
+      </c>
+      <c r="C578" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D578" s="1">
+        <v>2</v>
+      </c>
+      <c r="E578" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F578" s="1">
+        <v>6.38</v>
+      </c>
+      <c r="G578" s="14" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="579" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A579" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B579" t="s">
+        <v>10</v>
+      </c>
+      <c r="C579" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D579" s="1">
+        <v>1</v>
+      </c>
+      <c r="E579" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F579" s="1">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="580" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A580" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B580" t="s">
+        <v>10</v>
+      </c>
+      <c r="C580" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D580" s="1">
+        <v>6</v>
+      </c>
+      <c r="E580" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G580" s="14" t="s">
+        <v>448</v>
+      </c>
+      <c r="H580" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="581" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A581" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B581" t="s">
+        <v>10</v>
+      </c>
+      <c r="C581" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D581" s="1">
+        <v>9</v>
+      </c>
+      <c r="E581" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F581" s="1">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="582" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A582" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B582" t="s">
+        <v>10</v>
+      </c>
+      <c r="C582" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D582" s="1">
+        <v>19</v>
+      </c>
+      <c r="E582" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G582" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="H582" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="583" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A583" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B583" t="s">
+        <v>10</v>
+      </c>
+      <c r="C583" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D583" s="1">
+        <v>24</v>
+      </c>
+      <c r="E583" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F583" s="1">
+        <v>3.15</v>
+      </c>
+      <c r="G583" s="14" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="584" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A584" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B584" t="s">
+        <v>10</v>
+      </c>
+      <c r="C584" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D584" s="1">
+        <v>29</v>
+      </c>
+      <c r="E584" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F584" s="1">
+        <v>3.36</v>
+      </c>
+    </row>
+    <row r="585" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A585" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B585" t="s">
+        <v>10</v>
+      </c>
+      <c r="C585" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D585" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E585" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F585" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="G585" s="14" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="586" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A586" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B586" t="s">
+        <v>10</v>
+      </c>
+      <c r="C586" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D586" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="E586" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F586" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="G586" s="14" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="587" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A587" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B587" t="s">
+        <v>10</v>
+      </c>
+      <c r="C587" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D587" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E587" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F587" s="1">
+        <v>5.38</v>
+      </c>
+      <c r="G587" s="14" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="588" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A588" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B588" t="s">
+        <v>10</v>
+      </c>
+      <c r="C588" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D588" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="E588" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G588" s="14" t="s">
+        <v>365</v>
+      </c>
+      <c r="H588" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="589" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A589" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B589" t="s">
+        <v>18</v>
+      </c>
+      <c r="C589" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D589" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E589" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F589" s="1">
+        <v>1.77</v>
+      </c>
+      <c r="G589" s="14" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="590" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A590" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B590" t="s">
+        <v>18</v>
+      </c>
+      <c r="C590" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D590" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E590" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F590" s="1">
+        <v>2.0299999999999998</v>
+      </c>
+    </row>
+    <row r="591" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A591" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B591" t="s">
+        <v>10</v>
+      </c>
+      <c r="C591" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D591" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="E591" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G591" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="H591" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="592" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A592" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B592" t="s">
+        <v>10</v>
+      </c>
+      <c r="C592" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D592" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E592" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F592" s="1">
+        <v>0.56999999999999995</v>
+      </c>
+    </row>
+    <row r="593" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A593" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B593" t="s">
+        <v>10</v>
+      </c>
+      <c r="C593" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D593" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E593" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F593" s="1">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="594" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A594" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B594" t="s">
+        <v>18</v>
+      </c>
+      <c r="C594" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D594" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="E594" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G594" s="14" t="s">
+        <v>456</v>
+      </c>
+      <c r="H594" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="595" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A595" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B595" t="s">
+        <v>18</v>
+      </c>
+      <c r="C595" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D595" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="E595" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G595" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="H595" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="596" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A596" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B596" t="s">
+        <v>18</v>
+      </c>
+      <c r="C596" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="D596" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E596" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F596" s="1">
+        <v>3.28</v>
+      </c>
+      <c r="G596" s="14" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="597" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A597" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B597" t="s">
+        <v>18</v>
+      </c>
+      <c r="C597" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="D597" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="E597" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F597" s="1">
+        <v>6.07</v>
+      </c>
+    </row>
+    <row r="598" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A598" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B598" t="s">
+        <v>10</v>
+      </c>
+      <c r="C598" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="D598" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E598" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G598" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="H598" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="599" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A599" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B599" t="s">
+        <v>10</v>
+      </c>
+      <c r="C599" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="D599" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E599" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F599" s="1">
+        <v>3.72</v>
+      </c>
+      <c r="G599" s="14" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="600" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A600" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B600" t="s">
+        <v>10</v>
+      </c>
+      <c r="C600" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="D600" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E600" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G600" s="14" t="s">
+        <v>460</v>
+      </c>
+      <c r="H600" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="601" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A601" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B601" t="s">
+        <v>10</v>
+      </c>
+      <c r="C601" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D601" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E601" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F601" s="1">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="602" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A602" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B602" t="s">
+        <v>10</v>
+      </c>
+      <c r="C602" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D602" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="E602" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F602" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="G602" s="14" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="603" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A603" t="s">
+        <v>462</v>
+      </c>
+      <c r="B603" t="s">
+        <v>10</v>
+      </c>
+      <c r="C603" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D603" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E603" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F603" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G603" s="14" t="s">
+        <v>463</v>
+      </c>
+      <c r="H603" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="604" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A604" t="s">
+        <v>462</v>
+      </c>
+      <c r="B604" t="s">
+        <v>10</v>
+      </c>
+      <c r="C604" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D604" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E604" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F604" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="G604" s="14" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="605" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A605" t="s">
+        <v>462</v>
+      </c>
+      <c r="B605" t="s">
+        <v>10</v>
+      </c>
+      <c r="C605" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D605" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E605" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F605" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="G605" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="606" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A606" t="s">
+        <v>462</v>
+      </c>
+      <c r="B606" t="s">
+        <v>10</v>
+      </c>
+      <c r="C606" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D606" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E606" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F606" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="G606" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="607" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A607" t="s">
+        <v>462</v>
+      </c>
+      <c r="B607" t="s">
+        <v>271</v>
+      </c>
+      <c r="C607" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D607" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E607" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F607" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G607" s="14" t="s">
+        <v>468</v>
+      </c>
+      <c r="H607" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="608" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A608" t="s">
+        <v>462</v>
+      </c>
+      <c r="B608" t="s">
+        <v>18</v>
+      </c>
+      <c r="C608" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D608" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E608" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F608" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="G608" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="609" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A609" t="s">
+        <v>462</v>
+      </c>
+      <c r="B609" t="s">
+        <v>18</v>
+      </c>
+      <c r="C609" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D609" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E609" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F609" s="1">
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="610" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A610" t="s">
+        <v>462</v>
+      </c>
+      <c r="B610" t="s">
+        <v>18</v>
+      </c>
+      <c r="C610" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D610" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E610" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F610" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="G610" s="14" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="611" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A611" t="s">
+        <v>462</v>
+      </c>
+      <c r="B611" t="s">
+        <v>18</v>
+      </c>
+      <c r="C611" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D611" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E611" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F611" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G611" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H611" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="612" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A612" t="s">
+        <v>462</v>
+      </c>
+      <c r="B612" t="s">
+        <v>18</v>
+      </c>
+      <c r="C612" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D612" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E612" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F612" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G612" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H612" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="613" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A613" t="s">
+        <v>462</v>
+      </c>
+      <c r="B613" t="s">
+        <v>10</v>
+      </c>
+      <c r="C613" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D613" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E613" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F613" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="G613" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="614" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A614" t="s">
+        <v>462</v>
+      </c>
+      <c r="B614" t="s">
+        <v>18</v>
+      </c>
+      <c r="C614" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D614" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E614" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F614" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G614" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="H614" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="615" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A615" t="s">
+        <v>462</v>
+      </c>
+      <c r="B615" t="s">
+        <v>18</v>
+      </c>
+      <c r="C615" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D615" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E615" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F615" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G615" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="H615" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="616" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A616" t="s">
+        <v>485</v>
+      </c>
+      <c r="B616" t="s">
+        <v>10</v>
+      </c>
+      <c r="C616" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D616" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="E616" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G616" s="14" t="s">
+        <v>477</v>
+      </c>
+      <c r="H616" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="617" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A617" t="s">
+        <v>485</v>
+      </c>
+      <c r="B617" t="s">
+        <v>10</v>
+      </c>
+      <c r="C617" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D617" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="E617" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G617" s="14" t="s">
+        <v>478</v>
+      </c>
+      <c r="H617" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="618" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A618" t="s">
+        <v>485</v>
+      </c>
+      <c r="B618" t="s">
+        <v>10</v>
+      </c>
+      <c r="C618" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D618" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="E618" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G618" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="H618" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="619" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A619" t="s">
+        <v>485</v>
+      </c>
+      <c r="B619" t="s">
+        <v>10</v>
+      </c>
+      <c r="C619" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D619" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="E619" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G619" s="14" t="s">
+        <v>480</v>
+      </c>
+      <c r="H619" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="620" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A620" t="s">
+        <v>485</v>
+      </c>
+      <c r="B620" t="s">
+        <v>10</v>
+      </c>
+      <c r="C620" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D620" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="E620" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G620" s="14" t="s">
+        <v>480</v>
+      </c>
+      <c r="H620" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="621" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A621" t="s">
+        <v>485</v>
+      </c>
+      <c r="B621" t="s">
+        <v>18</v>
+      </c>
+      <c r="C621" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D621" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E621" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G621" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H621" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="622" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A622" t="s">
+        <v>485</v>
+      </c>
+      <c r="B622" t="s">
+        <v>18</v>
+      </c>
+      <c r="C622" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D622" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E622" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G622" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H622" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="623" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A623" t="s">
+        <v>485</v>
+      </c>
+      <c r="B623" t="s">
+        <v>18</v>
+      </c>
+      <c r="C623" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D623" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E623" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F623" s="1">
+        <v>5</v>
+      </c>
+      <c r="G623" s="14" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="624" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A624" t="s">
+        <v>485</v>
+      </c>
+      <c r="B624" t="s">
+        <v>18</v>
+      </c>
+      <c r="C624" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D624" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E624" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F624" s="1">
+        <v>3.3</v>
+      </c>
+      <c r="G624" s="14" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="625" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A625" t="s">
+        <v>485</v>
+      </c>
+      <c r="B625" t="s">
+        <v>18</v>
+      </c>
+      <c r="C625" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D625" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E625" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G625" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="H625" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="626" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A626" t="s">
+        <v>485</v>
+      </c>
+      <c r="B626" t="s">
+        <v>10</v>
+      </c>
+      <c r="C626" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D626" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="E626" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F626" s="1">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="627" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A627" t="s">
+        <v>485</v>
+      </c>
+      <c r="B627" t="s">
+        <v>10</v>
+      </c>
+      <c r="C627" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D627" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="E627" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G627" s="14" t="s">
+        <v>480</v>
+      </c>
+      <c r="H627" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="628" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A628" t="s">
+        <v>485</v>
+      </c>
+      <c r="B628" t="s">
+        <v>10</v>
+      </c>
+      <c r="C628" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D628" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="E628" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G628" s="14" t="s">
+        <v>483</v>
+      </c>
+      <c r="H628" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="629" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A629" t="s">
+        <v>485</v>
+      </c>
+      <c r="B629" t="s">
+        <v>10</v>
+      </c>
+      <c r="C629" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D629" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="E629" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F629" s="1">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="630" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A630" t="s">
+        <v>485</v>
+      </c>
+      <c r="B630" t="s">
+        <v>271</v>
+      </c>
+      <c r="C630" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D630" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="E630" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G630" s="14" t="s">
+        <v>484</v>
+      </c>
+      <c r="H630" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="631" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A631" t="s">
+        <v>485</v>
+      </c>
+      <c r="B631" t="s">
+        <v>18</v>
+      </c>
+      <c r="C631" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="D631" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E631" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F631" s="1">
+        <v>2.39</v>
+      </c>
+      <c r="G631" s="14" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="632" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A632" t="s">
+        <v>485</v>
+      </c>
+      <c r="B632" t="s">
+        <v>18</v>
+      </c>
+      <c r="C632" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="D632" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E632" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F632" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="G632" s="14" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="633" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A633" t="s">
+        <v>485</v>
+      </c>
+      <c r="B633" t="s">
+        <v>10</v>
+      </c>
+      <c r="C633" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="D633" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E633" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F633" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="G633" s="14" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="634" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A634" t="s">
+        <v>485</v>
+      </c>
+      <c r="B634" t="s">
+        <v>10</v>
+      </c>
+      <c r="C634" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="D634" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="E634" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F634" s="1">
+        <v>2.74</v>
+      </c>
+      <c r="G634" s="14" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="635" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A635" t="s">
+        <v>489</v>
+      </c>
+      <c r="B635" t="s">
+        <v>10</v>
+      </c>
+      <c r="C635" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D635" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E635" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F635" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="G635" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="636" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A636" t="s">
+        <v>489</v>
+      </c>
+      <c r="B636" t="s">
+        <v>10</v>
+      </c>
+      <c r="C636" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D636" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E636" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F636" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="G636" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="637" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A637" t="s">
+        <v>489</v>
+      </c>
+      <c r="B637" t="s">
+        <v>10</v>
+      </c>
+      <c r="C637" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D637" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E637" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F637" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="G637" s="14" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="638" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A638" t="s">
+        <v>489</v>
+      </c>
+      <c r="B638" t="s">
+        <v>10</v>
+      </c>
+      <c r="C638" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D638" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E638" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F638" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="G638" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="639" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A639" t="s">
+        <v>489</v>
+      </c>
+      <c r="B639" t="s">
+        <v>10</v>
+      </c>
+      <c r="C639" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D639" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E639" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F639" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="G639" s="14" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="640" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A640" t="s">
+        <v>489</v>
+      </c>
+      <c r="B640" t="s">
+        <v>18</v>
+      </c>
+      <c r="C640" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D640" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E640" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F640" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G640" s="14" t="s">
+        <v>497</v>
+      </c>
+      <c r="H640" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="641" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A641" t="s">
+        <v>489</v>
+      </c>
+      <c r="B641" t="s">
+        <v>18</v>
+      </c>
+      <c r="C641" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D641" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E641" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F641" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G641" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="H641" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="642" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A642" t="s">
+        <v>489</v>
+      </c>
+      <c r="B642" t="s">
+        <v>18</v>
+      </c>
+      <c r="C642" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D642" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E642" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F642" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G642" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H642" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="643" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A643" t="s">
+        <v>489</v>
+      </c>
+      <c r="B643" t="s">
+        <v>18</v>
+      </c>
+      <c r="C643" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D643" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E643" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F643" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G643" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="H643" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -13043,7 +16727,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Check column E" error="Free-text now allowed. Use column G &quot;Notes&quot; to free type." xr:uid="{E0C106E4-13F5-461C-BCAD-1CAD6FA54269}">
           <x14:formula1>
-            <xm:f>IF($E1048491="No", 'Data Dictionary'!$A$25:$A$30, 'Data Dictionary'!$A$32)</xm:f>
+            <xm:f>IF($E1048486="No", 'Data Dictionary'!$A$25:$A$30, 'Data Dictionary'!$A$32)</xm:f>
           </x14:formula1>
           <xm:sqref>H1</xm:sqref>
         </x14:dataValidation>
@@ -13051,7 +16735,7 @@
           <x14:formula1>
             <xm:f>IF($E433="No", 'Data Dictionary'!$A$25:$A$30, 'Data Dictionary'!$A$32)</xm:f>
           </x14:formula1>
-          <xm:sqref>H433:H672</xm:sqref>
+          <xm:sqref>H433:H667</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -13061,7 +16745,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{240BDDD7-65A5-4F9A-8645-E6E255B43C11}">
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:H181"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.75" customWidth="1"/>
@@ -16301,6 +19985,906 @@
       </c>
       <c r="G142" s="1">
         <v>7.04</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A143" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B143" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C143" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="D143" s="1">
+        <v>4</v>
+      </c>
+      <c r="E143" s="1">
+        <v>2</v>
+      </c>
+      <c r="F143" s="1">
+        <v>2</v>
+      </c>
+      <c r="G143" s="1">
+        <v>26.59</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A144" s="16">
+        <v>46302</v>
+      </c>
+      <c r="B144" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C144" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="D144" s="1">
+        <v>3</v>
+      </c>
+      <c r="E144" s="1">
+        <v>3</v>
+      </c>
+      <c r="F144" s="1">
+        <v>0</v>
+      </c>
+      <c r="G144" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A145" s="16">
+        <v>46303</v>
+      </c>
+      <c r="B145" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C145" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D145" s="1">
+        <v>4</v>
+      </c>
+      <c r="E145" s="1">
+        <v>2</v>
+      </c>
+      <c r="F145" s="1">
+        <v>2</v>
+      </c>
+      <c r="G145" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A146" s="16">
+        <v>46303</v>
+      </c>
+      <c r="B146" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C146" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D146" s="1">
+        <v>4</v>
+      </c>
+      <c r="E146" s="1">
+        <v>4</v>
+      </c>
+      <c r="F146" s="1">
+        <v>0</v>
+      </c>
+      <c r="G146" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A147" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B147" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C147" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D147" s="1">
+        <v>5</v>
+      </c>
+      <c r="E147" s="1">
+        <v>2</v>
+      </c>
+      <c r="F147" s="1">
+        <v>3</v>
+      </c>
+      <c r="G147" s="1">
+        <v>17.829999999999998</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A148" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B148" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C148" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="D148" s="1">
+        <v>2</v>
+      </c>
+      <c r="E148" s="1">
+        <v>2</v>
+      </c>
+      <c r="F148" s="1">
+        <v>0</v>
+      </c>
+      <c r="G148" s="1">
+        <v>20.41</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A149" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B149" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C149" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="D149" s="1">
+        <v>4</v>
+      </c>
+      <c r="E149" s="1">
+        <v>3</v>
+      </c>
+      <c r="F149" s="1">
+        <v>1</v>
+      </c>
+      <c r="G149" s="1">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A150" s="16">
+        <v>46304</v>
+      </c>
+      <c r="B150" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C150" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="D150" s="1">
+        <v>2</v>
+      </c>
+      <c r="E150" s="1">
+        <v>1</v>
+      </c>
+      <c r="F150" s="1">
+        <v>1</v>
+      </c>
+      <c r="G150" s="1">
+        <v>14.86</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A151" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B151" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C151" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="D151" s="1">
+        <v>4</v>
+      </c>
+      <c r="E151" s="1">
+        <v>3</v>
+      </c>
+      <c r="F151" s="1">
+        <v>1</v>
+      </c>
+      <c r="G151" s="1">
+        <v>19.059999999999999</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A152" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B152" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C152" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="D152" s="1">
+        <v>3</v>
+      </c>
+      <c r="E152" s="1">
+        <v>2</v>
+      </c>
+      <c r="F152" s="1">
+        <v>1</v>
+      </c>
+      <c r="G152" s="1">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A153" s="16">
+        <v>46305</v>
+      </c>
+      <c r="B153" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C153" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="D153" s="1">
+        <v>1</v>
+      </c>
+      <c r="E153" s="1">
+        <v>1</v>
+      </c>
+      <c r="F153" s="1">
+        <v>0</v>
+      </c>
+      <c r="G153" s="1">
+        <v>4.87</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A154" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B154" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C154" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="D154" s="1">
+        <v>2</v>
+      </c>
+      <c r="E154" s="1">
+        <v>2</v>
+      </c>
+      <c r="F154" s="1">
+        <v>0</v>
+      </c>
+      <c r="G154" s="1">
+        <v>13.75</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A155" s="16">
+        <v>46306</v>
+      </c>
+      <c r="B155" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C155" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="D155" s="1">
+        <v>6</v>
+      </c>
+      <c r="E155" s="1">
+        <v>3</v>
+      </c>
+      <c r="F155" s="1">
+        <v>3</v>
+      </c>
+      <c r="G155" s="1">
+        <v>44.15</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A156" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B156" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C156" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="D156" s="1">
+        <v>3</v>
+      </c>
+      <c r="E156" s="1">
+        <v>1</v>
+      </c>
+      <c r="F156" s="1">
+        <v>2</v>
+      </c>
+      <c r="G156" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A157" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B157" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C157" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="D157" s="1">
+        <v>4</v>
+      </c>
+      <c r="E157" s="1">
+        <v>4</v>
+      </c>
+      <c r="F157" s="1">
+        <v>0</v>
+      </c>
+      <c r="G157" s="1">
+        <v>35.07</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A158" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B158" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C158" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="D158" s="1">
+        <v>2</v>
+      </c>
+      <c r="E158" s="1">
+        <v>0</v>
+      </c>
+      <c r="F158" s="1">
+        <v>2</v>
+      </c>
+      <c r="G158" s="1">
+        <v>3.93</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A159" s="16">
+        <v>46307</v>
+      </c>
+      <c r="B159" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C159" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D159" s="1">
+        <v>2</v>
+      </c>
+      <c r="E159" s="1">
+        <v>2</v>
+      </c>
+      <c r="F159" s="1">
+        <v>0</v>
+      </c>
+      <c r="G159" s="1">
+        <v>34.119999999999997</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A160" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B160" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C160" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="D160" s="1">
+        <v>5</v>
+      </c>
+      <c r="E160" s="1">
+        <v>3</v>
+      </c>
+      <c r="F160" s="1">
+        <v>2</v>
+      </c>
+      <c r="G160" s="1">
+        <v>37.32</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A161" s="16">
+        <v>46308</v>
+      </c>
+      <c r="B161" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C161" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="D161" s="1">
+        <v>7</v>
+      </c>
+      <c r="E161" s="1">
+        <v>4</v>
+      </c>
+      <c r="F161" s="1">
+        <v>3</v>
+      </c>
+      <c r="G161" s="1">
+        <v>29.67</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A162" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B162" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C162" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D162" s="1">
+        <v>9</v>
+      </c>
+      <c r="E162" s="1">
+        <v>3</v>
+      </c>
+      <c r="F162" s="1">
+        <v>6</v>
+      </c>
+      <c r="G162" s="1">
+        <v>43.75</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A163" s="16">
+        <v>46309</v>
+      </c>
+      <c r="B163" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C163" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D163" s="1">
+        <v>3</v>
+      </c>
+      <c r="E163" s="1">
+        <v>3</v>
+      </c>
+      <c r="F163" s="1">
+        <v>0</v>
+      </c>
+      <c r="G163" s="1">
+        <v>31.41</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A164" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B164" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C164" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D164" s="1">
+        <v>2</v>
+      </c>
+      <c r="E164" s="1">
+        <v>2</v>
+      </c>
+      <c r="F164" s="1">
+        <v>0</v>
+      </c>
+      <c r="G164" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A165" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B165" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C165" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D165" s="1">
+        <v>2</v>
+      </c>
+      <c r="E165" s="1">
+        <v>1</v>
+      </c>
+      <c r="F165" s="1">
+        <v>1</v>
+      </c>
+      <c r="G165" s="1">
+        <v>8.74</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A166" s="16">
+        <v>46310</v>
+      </c>
+      <c r="B166" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C166" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D166" s="1">
+        <v>7</v>
+      </c>
+      <c r="E166" s="1">
+        <v>5</v>
+      </c>
+      <c r="F166" s="1">
+        <v>2</v>
+      </c>
+      <c r="G166" s="1">
+        <v>36.54</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A167" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B167" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C167" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D167" s="1">
+        <v>7</v>
+      </c>
+      <c r="E167" s="1">
+        <v>5</v>
+      </c>
+      <c r="F167" s="1">
+        <v>2</v>
+      </c>
+      <c r="G167" s="1">
+        <v>33.07</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A168" s="16">
+        <v>46311</v>
+      </c>
+      <c r="B168" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C168" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D168" s="1">
+        <v>4</v>
+      </c>
+      <c r="E168" s="1">
+        <v>2</v>
+      </c>
+      <c r="F168" s="1">
+        <v>2</v>
+      </c>
+      <c r="G168" s="1">
+        <v>18.149999999999999</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A169" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B169" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C169" s="11" t="s">
+        <v>369</v>
+      </c>
+      <c r="D169" s="1">
+        <v>2</v>
+      </c>
+      <c r="E169" s="1">
+        <v>2</v>
+      </c>
+      <c r="F169" s="1">
+        <v>0</v>
+      </c>
+      <c r="G169" s="1">
+        <v>10.98</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A170" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B170" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C170" s="11" t="s">
+        <v>369</v>
+      </c>
+      <c r="D170" s="1">
+        <v>3</v>
+      </c>
+      <c r="E170" s="1">
+        <v>1</v>
+      </c>
+      <c r="F170" s="1">
+        <v>2</v>
+      </c>
+      <c r="G170" s="1">
+        <v>8.07</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A171" s="16">
+        <v>46312</v>
+      </c>
+      <c r="B171" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C171" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="D171" s="1">
+        <v>2</v>
+      </c>
+      <c r="E171" s="1">
+        <v>2</v>
+      </c>
+      <c r="F171" s="1">
+        <v>0</v>
+      </c>
+      <c r="G171" s="1">
+        <v>4.79</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
+        <v>462</v>
+      </c>
+      <c r="B172" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C172" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D172" s="1">
+        <v>5</v>
+      </c>
+      <c r="E172" s="1">
+        <v>4</v>
+      </c>
+      <c r="F172" s="1">
+        <v>1</v>
+      </c>
+      <c r="G172" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
+        <v>462</v>
+      </c>
+      <c r="B173" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C173" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D173" s="1">
+        <v>1</v>
+      </c>
+      <c r="E173" s="1">
+        <v>0</v>
+      </c>
+      <c r="F173" s="1">
+        <v>1</v>
+      </c>
+      <c r="G173" s="1" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
+        <v>462</v>
+      </c>
+      <c r="B174" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C174" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D174" s="1">
+        <v>7</v>
+      </c>
+      <c r="E174" s="1">
+        <v>3</v>
+      </c>
+      <c r="F174" s="1">
+        <v>4</v>
+      </c>
+      <c r="G174" s="1" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A175" t="s">
+        <v>485</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C175" s="17">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D175" s="8">
+        <v>9</v>
+      </c>
+      <c r="E175" s="8">
+        <v>2</v>
+      </c>
+      <c r="F175" s="8">
+        <v>7</v>
+      </c>
+      <c r="G175" s="8">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="H175" s="7"/>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A176" t="s">
+        <v>485</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C176" s="17">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D176" s="8">
+        <v>5</v>
+      </c>
+      <c r="E176" s="8">
+        <v>2</v>
+      </c>
+      <c r="F176" s="8">
+        <v>3</v>
+      </c>
+      <c r="G176" s="8">
+        <v>21.23</v>
+      </c>
+      <c r="H176" s="7"/>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A177" t="s">
+        <v>485</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="C177" s="17">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D177" s="8">
+        <v>1</v>
+      </c>
+      <c r="E177" s="8">
+        <v>0</v>
+      </c>
+      <c r="F177" s="8">
+        <v>1</v>
+      </c>
+      <c r="G177" s="8">
+        <v>0.94</v>
+      </c>
+      <c r="H177" s="7"/>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A178" s="16">
+        <v>46315</v>
+      </c>
+      <c r="B178" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C178" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="D178" s="1">
+        <v>2</v>
+      </c>
+      <c r="E178" s="1">
+        <v>2</v>
+      </c>
+      <c r="F178" s="1">
+        <v>0</v>
+      </c>
+      <c r="G178" s="1">
+        <v>10.37</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A179" s="16">
+        <v>46315</v>
+      </c>
+      <c r="B179" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C179" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="D179" s="1">
+        <v>2</v>
+      </c>
+      <c r="E179" s="1">
+        <v>2</v>
+      </c>
+      <c r="F179" s="1">
+        <v>0</v>
+      </c>
+      <c r="G179" s="1">
+        <v>10.54</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A180" t="s">
+        <v>489</v>
+      </c>
+      <c r="B180" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C180" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D180" s="1">
+        <v>5</v>
+      </c>
+      <c r="E180" s="1">
+        <v>5</v>
+      </c>
+      <c r="F180" s="1">
+        <v>0</v>
+      </c>
+      <c r="G180" s="1" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A181" t="s">
+        <v>489</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C181" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D181" s="1">
+        <v>4</v>
+      </c>
+      <c r="E181" s="1">
+        <v>0</v>
+      </c>
+      <c r="F181" s="1">
+        <v>4</v>
+      </c>
+      <c r="G181" s="1" t="s">
+        <v>499</v>
       </c>
     </row>
   </sheetData>
@@ -16347,7 +20931,7 @@
         <v>86</v>
       </c>
       <c r="B5" s="2" cm="1">
-        <f t="array" ref="B5">MIN(IF(Patient_Log!F16:F1029&gt;=1,Patient_Log!F16:F1029))</f>
+        <f t="array" ref="B5">MIN(IF(Patient_Log!F16:F1024&gt;=1,Patient_Log!F16:F1024))</f>
         <v>1</v>
       </c>
     </row>
@@ -16356,7 +20940,7 @@
         <v>87</v>
       </c>
       <c r="B6" s="1" cm="1">
-        <f t="array" ref="B6">MAX(IF(Patient_Log!F16:F1029&gt;=1,Patient_Log!F16:F1029))</f>
+        <f t="array" ref="B6">MAX(IF(Patient_Log!F16:F1024&gt;=1,Patient_Log!F16:F1024))</f>
         <v>47.21</v>
       </c>
     </row>
@@ -16365,8 +20949,8 @@
         <v>88</v>
       </c>
       <c r="B7" s="2">
-        <f>AVERAGEIF(Patient_Log!F16:F1029,"&lt;&gt;0")</f>
-        <v>5.7113782051282049</v>
+        <f>AVERAGEIF(Patient_Log!F16:F1024,"&lt;&gt;0")</f>
+        <v>5.5995607235142115</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -16377,8 +20961,8 @@
         <v>80</v>
       </c>
       <c r="B9" s="1">
-        <f>SUM(Unit_Log!E2:E997)</f>
-        <v>371</v>
+        <f>SUM(Unit_Log!E2:E994)</f>
+        <v>461</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -16400,7 +20984,7 @@
         <v>90</v>
       </c>
       <c r="B12" s="1" cm="1">
-        <f t="array" ref="B12">MIN(IF(Unit_Log!G2:G997&gt;=1,Unit_Log!G2:G997))</f>
+        <f t="array" ref="B12">MIN(IF(Unit_Log!G2:G994&gt;=1,Unit_Log!G2:G994))</f>
         <v>1</v>
       </c>
     </row>
@@ -16409,7 +20993,7 @@
         <v>91</v>
       </c>
       <c r="B13" s="1" cm="1">
-        <f t="array" ref="B13">MAX(IF(Unit_Log!G8:G997&gt;=1,Unit_Log!G8:G997))</f>
+        <f t="array" ref="B13">MAX(IF(Unit_Log!G8:G994&gt;=1,Unit_Log!G8:G994))</f>
         <v>78.23</v>
       </c>
     </row>

</xml_diff>